<commit_message>
data sampai halaman 12
</commit_message>
<xml_diff>
--- a/public/kotoba_mokuzai.xlsx
+++ b/public/kotoba_mokuzai.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\mokuzai_flashcard\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36E6D1DE-0754-4316-A2BC-314F5387D0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B2E126-30C3-4CBC-A66C-AFD5601B08B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1678" uniqueCount="1253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2332" uniqueCount="1669">
   <si>
     <t>第１章</t>
   </si>
@@ -3779,6 +3779,1254 @@
   </si>
   <si>
     <t>arti</t>
+  </si>
+  <si>
+    <t>強さ</t>
+  </si>
+  <si>
+    <t>つよさ</t>
+  </si>
+  <si>
+    <t>kekuatan</t>
+  </si>
+  <si>
+    <t>力</t>
+  </si>
+  <si>
+    <t>ちから</t>
+  </si>
+  <si>
+    <t>gaya, tenaga</t>
+  </si>
+  <si>
+    <t>加える</t>
+  </si>
+  <si>
+    <t>くわえる</t>
+  </si>
+  <si>
+    <t>memberikan, menerapkan</t>
+  </si>
+  <si>
+    <t>方法</t>
+  </si>
+  <si>
+    <t>ほうほう</t>
+  </si>
+  <si>
+    <t>metode, cara</t>
+  </si>
+  <si>
+    <t>方向</t>
+  </si>
+  <si>
+    <t>ほうこう</t>
+  </si>
+  <si>
+    <t>arah</t>
+  </si>
+  <si>
+    <t>圧縮強さ</t>
+  </si>
+  <si>
+    <t>あっしゅくつよさ</t>
+  </si>
+  <si>
+    <t>kekuatan tekan</t>
+  </si>
+  <si>
+    <t>引張強さ</t>
+  </si>
+  <si>
+    <t>ひっぱりつよさ</t>
+  </si>
+  <si>
+    <t>kekuatan tarik</t>
+  </si>
+  <si>
+    <t>曲げ強さ</t>
+  </si>
+  <si>
+    <t>まげつよさ</t>
+  </si>
+  <si>
+    <t>kekuatan lentur</t>
+  </si>
+  <si>
+    <t>せん断強さ</t>
+  </si>
+  <si>
+    <t>せんだんつよさ</t>
+  </si>
+  <si>
+    <t>kekuatan geser</t>
+  </si>
+  <si>
+    <t>割裂強さ</t>
+  </si>
+  <si>
+    <t>かつれつつよさ</t>
+  </si>
+  <si>
+    <t>kekuatan belah</t>
+  </si>
+  <si>
+    <t>表す</t>
+  </si>
+  <si>
+    <t>あらわす</t>
+  </si>
+  <si>
+    <t>menyatakan, menunjukkan</t>
+  </si>
+  <si>
+    <t>berikut</t>
+  </si>
+  <si>
+    <t>関係する</t>
+  </si>
+  <si>
+    <t>かんけいする</t>
+  </si>
+  <si>
+    <t>berhubungan dengan</t>
+  </si>
+  <si>
+    <t>密度</t>
+  </si>
+  <si>
+    <t>みつど</t>
+  </si>
+  <si>
+    <t>densitas, massa jenis</t>
+  </si>
+  <si>
+    <t>一般に</t>
+  </si>
+  <si>
+    <t>いっぱんに</t>
+  </si>
+  <si>
+    <t>pada umumnya</t>
+  </si>
+  <si>
+    <t>densitas</t>
+  </si>
+  <si>
+    <t>大きい</t>
+  </si>
+  <si>
+    <t>おおきい</t>
+  </si>
+  <si>
+    <t>besar</t>
+  </si>
+  <si>
+    <t>大きくなる</t>
+  </si>
+  <si>
+    <t>おおきくなる</t>
+  </si>
+  <si>
+    <t>menjadi lebih besar</t>
+  </si>
+  <si>
+    <t>数％</t>
+  </si>
+  <si>
+    <t>すうパーセント</t>
+  </si>
+  <si>
+    <t>beberapa persen</t>
+  </si>
+  <si>
+    <t>前後</t>
+  </si>
+  <si>
+    <t>ぜんご</t>
+  </si>
+  <si>
+    <t>menjadi paling besar</t>
+  </si>
+  <si>
+    <t>繊維飽和点</t>
+  </si>
+  <si>
+    <t>せんいほうわてん</t>
+  </si>
+  <si>
+    <t>titik jenuh serat</t>
+  </si>
+  <si>
+    <t>以上</t>
+  </si>
+  <si>
+    <t>いじょう</t>
+  </si>
+  <si>
+    <t>lebih dari</t>
+  </si>
+  <si>
+    <t>一定</t>
+  </si>
+  <si>
+    <t>いってい</t>
+  </si>
+  <si>
+    <t>tetap, konstan</t>
+  </si>
+  <si>
+    <t>arah serat</t>
+  </si>
+  <si>
+    <t>圧縮</t>
+  </si>
+  <si>
+    <t>あっしゅく</t>
+  </si>
+  <si>
+    <t>kompresi, tekan</t>
+  </si>
+  <si>
+    <t>強い</t>
+  </si>
+  <si>
+    <t>つよい</t>
+  </si>
+  <si>
+    <t>kuat</t>
+  </si>
+  <si>
+    <t>横方向</t>
+  </si>
+  <si>
+    <t>よこほうこう</t>
+  </si>
+  <si>
+    <t>arah melintang</t>
+  </si>
+  <si>
+    <t>半径方向</t>
+  </si>
+  <si>
+    <t>はんけいほうこう</t>
+  </si>
+  <si>
+    <t>arah radial</t>
+  </si>
+  <si>
+    <t>外</t>
+  </si>
+  <si>
+    <t>そと</t>
+  </si>
+  <si>
+    <t>luar</t>
+  </si>
+  <si>
+    <t>向かう</t>
+  </si>
+  <si>
+    <t>むかう</t>
+  </si>
+  <si>
+    <t>menuju</t>
+  </si>
+  <si>
+    <t>lebih... (dalam perbandingan)</t>
+  </si>
+  <si>
+    <t>arah tangensial</t>
+  </si>
+  <si>
+    <t>lingkaran tahun</t>
+  </si>
+  <si>
+    <t>接する</t>
+  </si>
+  <si>
+    <t>せっする</t>
+  </si>
+  <si>
+    <t>bersentuhan, menyinggung</t>
+  </si>
+  <si>
+    <t>節</t>
+  </si>
+  <si>
+    <t>ふし</t>
+  </si>
+  <si>
+    <t>mata kayu, simpul kayu</t>
+  </si>
+  <si>
+    <t>mata kayu</t>
+  </si>
+  <si>
+    <t>周辺</t>
+  </si>
+  <si>
+    <t>しゅうへん</t>
+  </si>
+  <si>
+    <t>繊維</t>
+  </si>
+  <si>
+    <t>せんい</t>
+  </si>
+  <si>
+    <t>serat</t>
+  </si>
+  <si>
+    <t>乱れ</t>
+  </si>
+  <si>
+    <t>みだれ</t>
+  </si>
+  <si>
+    <t>ketidakteraturan</t>
+  </si>
+  <si>
+    <t>小さくなる</t>
+  </si>
+  <si>
+    <t>ちいさくなる</t>
+  </si>
+  <si>
+    <t>menjadi lebih kecil</t>
+  </si>
+  <si>
+    <t>圧縮強度</t>
+  </si>
+  <si>
+    <t>あっしゅくきょうど</t>
+  </si>
+  <si>
+    <t>kuat tekan</t>
+  </si>
+  <si>
+    <t>引張強度</t>
+  </si>
+  <si>
+    <t>ひっぱりきょうど</t>
+  </si>
+  <si>
+    <t>kuat tarik</t>
+  </si>
+  <si>
+    <t>影響</t>
+  </si>
+  <si>
+    <t>えいきょう</t>
+  </si>
+  <si>
+    <t>pengaruh</t>
+  </si>
+  <si>
+    <t>及ぼす</t>
+  </si>
+  <si>
+    <t>およぼす</t>
+  </si>
+  <si>
+    <t>memberikan, menimbulkan</t>
+  </si>
+  <si>
+    <t>温度</t>
+  </si>
+  <si>
+    <t>おんど</t>
+  </si>
+  <si>
+    <t>suhu</t>
+  </si>
+  <si>
+    <t>樹幹内</t>
+  </si>
+  <si>
+    <t>じゅかんない</t>
+  </si>
+  <si>
+    <t>di dalam batang pohon</t>
+  </si>
+  <si>
+    <t>部位</t>
+  </si>
+  <si>
+    <t>ぶい</t>
+  </si>
+  <si>
+    <t>bagian, posisi</t>
+  </si>
+  <si>
+    <t>晩材率</t>
+  </si>
+  <si>
+    <t>ばんざいりつ</t>
+  </si>
+  <si>
+    <t>persentase kayu akhir (latewood)</t>
+  </si>
+  <si>
+    <t>平均年輪幅</t>
+  </si>
+  <si>
+    <t>へいきんねんりんはば</t>
+  </si>
+  <si>
+    <t>lebar rata-rata lingkaran tahun</t>
+  </si>
+  <si>
+    <t>寸法</t>
+  </si>
+  <si>
+    <t>すんぽう</t>
+  </si>
+  <si>
+    <t>dimensi, ukuran</t>
+  </si>
+  <si>
+    <t>あて材</t>
+  </si>
+  <si>
+    <t>あてざい</t>
+  </si>
+  <si>
+    <t>kayu reaksi (reaction wood)</t>
+  </si>
+  <si>
+    <t>腐れ</t>
+  </si>
+  <si>
+    <t>くされ</t>
+  </si>
+  <si>
+    <t>pembusukan</t>
+  </si>
+  <si>
+    <t>cacat, kelemahan</t>
+  </si>
+  <si>
+    <t>影響する</t>
+  </si>
+  <si>
+    <t>えいきょうする</t>
+  </si>
+  <si>
+    <t>mempengaruhi</t>
+  </si>
+  <si>
+    <t>作業安全</t>
+  </si>
+  <si>
+    <t>さぎょうあんぜん</t>
+  </si>
+  <si>
+    <t>keselamatan kerja</t>
+  </si>
+  <si>
+    <t>industri kayu</t>
+  </si>
+  <si>
+    <t>労働災害</t>
+  </si>
+  <si>
+    <t>ろうどうさいがい</t>
+  </si>
+  <si>
+    <t>kecelakaan kerja</t>
+  </si>
+  <si>
+    <t>発生状況</t>
+  </si>
+  <si>
+    <t>はっせいじょうきょう</t>
+  </si>
+  <si>
+    <t>kondisi/keadaan terjadinya</t>
+  </si>
+  <si>
+    <t>死傷者数</t>
+  </si>
+  <si>
+    <t>ししょうしゃすう</t>
+  </si>
+  <si>
+    <t>jumlah korban meninggal dan luka</t>
+  </si>
+  <si>
+    <t>年間</t>
+  </si>
+  <si>
+    <t>ねんかん</t>
+  </si>
+  <si>
+    <t>per tahun</t>
+  </si>
+  <si>
+    <t>件</t>
+  </si>
+  <si>
+    <t>けん</t>
+  </si>
+  <si>
+    <t>kasus, kejadian</t>
+  </si>
+  <si>
+    <t>死亡災害</t>
+  </si>
+  <si>
+    <t>しぼうさいがい</t>
+  </si>
+  <si>
+    <t>kecelakaan fatal</t>
+  </si>
+  <si>
+    <t>kasus</t>
+  </si>
+  <si>
+    <t>安全</t>
+  </si>
+  <si>
+    <t>あんぜん</t>
+  </si>
+  <si>
+    <t>keamanan, keselamatan</t>
+  </si>
+  <si>
+    <t>安全対策</t>
+  </si>
+  <si>
+    <t>あんぜんたいさく</t>
+  </si>
+  <si>
+    <t>tindakan keselamatan</t>
+  </si>
+  <si>
+    <t>推進</t>
+  </si>
+  <si>
+    <t>すいしん</t>
+  </si>
+  <si>
+    <t>pendorongan, pengembangan</t>
+  </si>
+  <si>
+    <t>件数</t>
+  </si>
+  <si>
+    <t>けんすう</t>
+  </si>
+  <si>
+    <t>jumlah kasus</t>
+  </si>
+  <si>
+    <t>減る</t>
+  </si>
+  <si>
+    <t>へる</t>
+  </si>
+  <si>
+    <t>berkurang</t>
+  </si>
+  <si>
+    <t>発生率</t>
+  </si>
+  <si>
+    <t>はっせいりつ</t>
+  </si>
+  <si>
+    <t>tingkat kejadian</t>
+  </si>
+  <si>
+    <t>他</t>
+  </si>
+  <si>
+    <t>ほか</t>
+  </si>
+  <si>
+    <t>lain</t>
+  </si>
+  <si>
+    <t>倍</t>
+  </si>
+  <si>
+    <t>ばい</t>
+  </si>
+  <si>
+    <t>kali lipat</t>
+  </si>
+  <si>
+    <t>高い</t>
+  </si>
+  <si>
+    <t>たかい</t>
+  </si>
+  <si>
+    <t>tinggi</t>
+  </si>
+  <si>
+    <t>改善</t>
+  </si>
+  <si>
+    <t>かいぜん</t>
+  </si>
+  <si>
+    <t>perbaikan</t>
+  </si>
+  <si>
+    <t>事故</t>
+  </si>
+  <si>
+    <t>じこ</t>
+  </si>
+  <si>
+    <t>kecelakaan</t>
+  </si>
+  <si>
+    <t>約半分</t>
+  </si>
+  <si>
+    <t>やくはんぶん</t>
+  </si>
+  <si>
+    <t>sekitar setengah</t>
+  </si>
+  <si>
+    <t>切れ</t>
+  </si>
+  <si>
+    <t>きれ</t>
+  </si>
+  <si>
+    <t>luka karena benda tajam/terpotong</t>
+  </si>
+  <si>
+    <t>こすれ</t>
+  </si>
+  <si>
+    <t>gesekan</t>
+  </si>
+  <si>
+    <t>挟まれ</t>
+  </si>
+  <si>
+    <t>はさまれ</t>
+  </si>
+  <si>
+    <t>terjepit</t>
+  </si>
+  <si>
+    <t>巻き込まれ</t>
+  </si>
+  <si>
+    <t>まきこまれ</t>
+  </si>
+  <si>
+    <t>tersangkut/terseret ke mesin</t>
+  </si>
+  <si>
+    <t>木材加工</t>
+  </si>
+  <si>
+    <t>もくざいかこう</t>
+  </si>
+  <si>
+    <t>pengolahan kayu</t>
+  </si>
+  <si>
+    <t>作業</t>
+  </si>
+  <si>
+    <t>さぎょう</t>
+  </si>
+  <si>
+    <t>pekerjaan, operasi kerja</t>
+  </si>
+  <si>
+    <t>発生する</t>
+  </si>
+  <si>
+    <t>はっせいする</t>
+  </si>
+  <si>
+    <t>terjadi</t>
+  </si>
+  <si>
+    <t>高速</t>
+  </si>
+  <si>
+    <t>こうそく</t>
+  </si>
+  <si>
+    <t>berkecepatan tinggi</t>
+  </si>
+  <si>
+    <t>回転する</t>
+  </si>
+  <si>
+    <t>かいてんする</t>
+  </si>
+  <si>
+    <t>berputar</t>
+  </si>
+  <si>
+    <t>工具</t>
+  </si>
+  <si>
+    <t>こうぐ</t>
+  </si>
+  <si>
+    <t>alat kerja, perkakas</t>
+  </si>
+  <si>
+    <t>触れる</t>
+  </si>
+  <si>
+    <t>ふれる</t>
+  </si>
+  <si>
+    <t>menyentuh</t>
+  </si>
+  <si>
+    <t>alat kerja</t>
+  </si>
+  <si>
+    <t>putaran</t>
+  </si>
+  <si>
+    <t>bahan kayu</t>
+  </si>
+  <si>
+    <t>送る</t>
+  </si>
+  <si>
+    <t>おくる</t>
+  </si>
+  <si>
+    <t>mengirim, mendorong</t>
+  </si>
+  <si>
+    <t>装置</t>
+  </si>
+  <si>
+    <t>そうち</t>
+  </si>
+  <si>
+    <t>perangkat, alat</t>
+  </si>
+  <si>
+    <t>起きる</t>
+  </si>
+  <si>
+    <t>おきる</t>
+  </si>
+  <si>
+    <t>pekerjaan</t>
+  </si>
+  <si>
+    <t>十分</t>
+  </si>
+  <si>
+    <t>じゅうぶん</t>
+  </si>
+  <si>
+    <t>cukup, memadai</t>
+  </si>
+  <si>
+    <t>注意</t>
+  </si>
+  <si>
+    <t>ちゅうい</t>
+  </si>
+  <si>
+    <t>perhatian, kewaspadaan</t>
+  </si>
+  <si>
+    <t>diperlukan</t>
+  </si>
+  <si>
+    <t>lainnya</t>
+  </si>
+  <si>
+    <t>terseret/tertarik ke mesin</t>
+  </si>
+  <si>
+    <t>飛来</t>
+  </si>
+  <si>
+    <t>ひらい</t>
+  </si>
+  <si>
+    <t>benda yang terbang/meluncur</t>
+  </si>
+  <si>
+    <t>落下</t>
+  </si>
+  <si>
+    <t>らっか</t>
+  </si>
+  <si>
+    <t>jatuh</t>
+  </si>
+  <si>
+    <t>転倒</t>
+  </si>
+  <si>
+    <t>てんとう</t>
+  </si>
+  <si>
+    <t>terjatuh</t>
+  </si>
+  <si>
+    <t>墜落</t>
+  </si>
+  <si>
+    <t>ついらく</t>
+  </si>
+  <si>
+    <t>jatuh dari ketinggian</t>
+  </si>
+  <si>
+    <t>転落</t>
+  </si>
+  <si>
+    <t>てんらく</t>
+  </si>
+  <si>
+    <t>terperosok/jatuh</t>
+  </si>
+  <si>
+    <t>terpotong</t>
+  </si>
+  <si>
+    <t>tergesek</t>
+  </si>
+  <si>
+    <t>型別</t>
+  </si>
+  <si>
+    <t>かたべつ</t>
+  </si>
+  <si>
+    <t>berdasarkan jenis</t>
+  </si>
+  <si>
+    <t>keselamatan, aman</t>
+  </si>
+  <si>
+    <t>配慮</t>
+  </si>
+  <si>
+    <t>はいりょ</t>
+  </si>
+  <si>
+    <t>perhatian, pertimbangan</t>
+  </si>
+  <si>
+    <t>服装</t>
+  </si>
+  <si>
+    <t>ふくそう</t>
+  </si>
+  <si>
+    <t>pakaian</t>
+  </si>
+  <si>
+    <t>keselamatan</t>
+  </si>
+  <si>
+    <t>pekerjaan, aktivitas kerja</t>
+  </si>
+  <si>
+    <t>内容</t>
+  </si>
+  <si>
+    <t>ないよう</t>
+  </si>
+  <si>
+    <t>isi, jenis pekerjaan</t>
+  </si>
+  <si>
+    <t>合わせる</t>
+  </si>
+  <si>
+    <t>あわせる</t>
+  </si>
+  <si>
+    <t>menyesuaikan</t>
+  </si>
+  <si>
+    <t>選ぶ</t>
+  </si>
+  <si>
+    <t>えらぶ</t>
+  </si>
+  <si>
+    <t>memilih</t>
+  </si>
+  <si>
+    <t>perlu</t>
+  </si>
+  <si>
+    <t>袖締まり</t>
+  </si>
+  <si>
+    <t>そでじまり</t>
+  </si>
+  <si>
+    <t>bagian ujung lengan baju yang pas/tidak longgar</t>
+  </si>
+  <si>
+    <t>裾締まり</t>
+  </si>
+  <si>
+    <t>すそじまり</t>
+  </si>
+  <si>
+    <t>bagian bawah pakaian yang pas/tidak longgar</t>
+  </si>
+  <si>
+    <t>作業服</t>
+  </si>
+  <si>
+    <t>さぎょうふく</t>
+  </si>
+  <si>
+    <t>pakaian kerja</t>
+  </si>
+  <si>
+    <t>着用</t>
+  </si>
+  <si>
+    <t>ちゃくよう</t>
+  </si>
+  <si>
+    <t>memakai</t>
+  </si>
+  <si>
+    <t>特に</t>
+  </si>
+  <si>
+    <t>とくに</t>
+  </si>
+  <si>
+    <t>歯</t>
+  </si>
+  <si>
+    <t>は</t>
+  </si>
+  <si>
+    <t>mata gergaji</t>
+  </si>
+  <si>
+    <t>巻き込まれる</t>
+  </si>
+  <si>
+    <t>まきこまれる</t>
+  </si>
+  <si>
+    <t>terseret/tertarik ke dalam mesin</t>
+  </si>
+  <si>
+    <t>衣類</t>
+  </si>
+  <si>
+    <t>いるい</t>
+  </si>
+  <si>
+    <t>紐</t>
+  </si>
+  <si>
+    <t>ひも</t>
+  </si>
+  <si>
+    <t>tali</t>
+  </si>
+  <si>
+    <t>perhatian, waspada</t>
+  </si>
+  <si>
+    <t>手袋</t>
+  </si>
+  <si>
+    <t>てぶくろ</t>
+  </si>
+  <si>
+    <t>sarung tangan</t>
+  </si>
+  <si>
+    <t>前掛け</t>
+  </si>
+  <si>
+    <t>まえかけ</t>
+  </si>
+  <si>
+    <t>celemek/apron</t>
+  </si>
+  <si>
+    <t>手ぬぐい</t>
+  </si>
+  <si>
+    <t>てぬぐい</t>
+  </si>
+  <si>
+    <t>handuk kain tradisional Jepang</t>
+  </si>
+  <si>
+    <t>作業帽</t>
+  </si>
+  <si>
+    <t>さぎょうぼう</t>
+  </si>
+  <si>
+    <t>topi kerja</t>
+  </si>
+  <si>
+    <t>保護</t>
+  </si>
+  <si>
+    <t>ほご</t>
+  </si>
+  <si>
+    <t>perlindungan</t>
+  </si>
+  <si>
+    <t>保護メガネ</t>
+  </si>
+  <si>
+    <t>ほごメガネ</t>
+  </si>
+  <si>
+    <t>kacamata pelindung</t>
+  </si>
+  <si>
+    <t>マスク</t>
+  </si>
+  <si>
+    <t>masker</t>
+  </si>
+  <si>
+    <t>安全靴</t>
+  </si>
+  <si>
+    <t>あんぜんぐつ</t>
+  </si>
+  <si>
+    <t>sepatu keselamatan</t>
+  </si>
+  <si>
+    <t>耳栓</t>
+  </si>
+  <si>
+    <t>みみせん</t>
+  </si>
+  <si>
+    <t>penyumbat telinga</t>
+  </si>
+  <si>
+    <t>保護具</t>
+  </si>
+  <si>
+    <t>ほごぐ</t>
+  </si>
+  <si>
+    <t>alat pelindung diri (APD)</t>
+  </si>
+  <si>
+    <t>正しく</t>
+  </si>
+  <si>
+    <t>ただしく</t>
+  </si>
+  <si>
+    <t>dengan benar</t>
+  </si>
+  <si>
+    <t>着用する</t>
+  </si>
+  <si>
+    <t>ちゃくようする</t>
+  </si>
+  <si>
+    <t>リスクアセスメント</t>
+  </si>
+  <si>
+    <t>penilaian risiko (risk assessment)</t>
+  </si>
+  <si>
+    <t>作業場</t>
+  </si>
+  <si>
+    <t>さぎょうじょう</t>
+  </si>
+  <si>
+    <t>tempat kerja</t>
+  </si>
+  <si>
+    <t>危ない</t>
+  </si>
+  <si>
+    <t>あぶない</t>
+  </si>
+  <si>
+    <t>berbahaya</t>
+  </si>
+  <si>
+    <t>見つけ出す</t>
+  </si>
+  <si>
+    <t>みつけだす</t>
+  </si>
+  <si>
+    <t>menemukan</t>
+  </si>
+  <si>
+    <t>被害</t>
+  </si>
+  <si>
+    <t>ひがい</t>
+  </si>
+  <si>
+    <t>kerugian, dampak</t>
+  </si>
+  <si>
+    <t>大きさ</t>
+  </si>
+  <si>
+    <t>おおきさ</t>
+  </si>
+  <si>
+    <t>besarnya</t>
+  </si>
+  <si>
+    <t>災害</t>
+  </si>
+  <si>
+    <t>さいがい</t>
+  </si>
+  <si>
+    <t>kecelakaan, bencana</t>
+  </si>
+  <si>
+    <t>可能性</t>
+  </si>
+  <si>
+    <t>かのうせい</t>
+  </si>
+  <si>
+    <t>kemungkinan</t>
+  </si>
+  <si>
+    <t>高さ</t>
+  </si>
+  <si>
+    <t>たかさ</t>
+  </si>
+  <si>
+    <t>tingkat ketinggian</t>
+  </si>
+  <si>
+    <t>優先度</t>
+  </si>
+  <si>
+    <t>ゆうせんど</t>
+  </si>
+  <si>
+    <t>tingkat prioritas</t>
+  </si>
+  <si>
+    <t>判定する</t>
+  </si>
+  <si>
+    <t>はんていする</t>
+  </si>
+  <si>
+    <t>menilai, menentukan</t>
+  </si>
+  <si>
+    <t>prioritas</t>
+  </si>
+  <si>
+    <t>減らす</t>
+  </si>
+  <si>
+    <t>へらす</t>
+  </si>
+  <si>
+    <t>mengurangi</t>
+  </si>
+  <si>
+    <t>検討する</t>
+  </si>
+  <si>
+    <t>けんとうする</t>
+  </si>
+  <si>
+    <t>mempertimbangkan, mengkaji</t>
+  </si>
+  <si>
+    <t>明確化</t>
+  </si>
+  <si>
+    <t>めいかくか</t>
+  </si>
+  <si>
+    <t>memperjelas, klarifikasi</t>
+  </si>
+  <si>
+    <t>働く</t>
+  </si>
+  <si>
+    <t>はたらく</t>
+  </si>
+  <si>
+    <t>bekerja</t>
+  </si>
+  <si>
+    <t>人たち</t>
+  </si>
+  <si>
+    <t>ひとたち</t>
+  </si>
+  <si>
+    <t>orang-orang</t>
+  </si>
+  <si>
+    <t>認識</t>
+  </si>
+  <si>
+    <t>にんしき</t>
+  </si>
+  <si>
+    <t>kesadaran, pemahaman</t>
+  </si>
+  <si>
+    <t>共有</t>
+  </si>
+  <si>
+    <t>きょうゆう</t>
+  </si>
+  <si>
+    <t>berbagi, saling memahami</t>
+  </si>
+  <si>
+    <t>効果</t>
+  </si>
+  <si>
+    <t>こうか</t>
+  </si>
+  <si>
+    <t>efek, manfaat</t>
+  </si>
+  <si>
+    <t>期待する</t>
+  </si>
+  <si>
+    <t>きたいする</t>
+  </si>
+  <si>
+    <t>mengharapkan</t>
   </si>
 </sst>
 </file>
@@ -3865,7 +5113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3882,6 +5130,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4100,7 +5351,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G559"/>
+  <dimension ref="A1:G777"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="33" customWidth="1"/>
@@ -4122,7 +5373,7 @@
         <v>1252</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" ht="13">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -4136,7 +5387,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" ht="13">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -4150,7 +5401,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" ht="13">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -4164,7 +5415,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" ht="13">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -4178,7 +5429,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" ht="13">
       <c r="A6" s="1">
         <v>1</v>
       </c>
@@ -4192,7 +5443,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" ht="13">
       <c r="A7" s="1">
         <v>1</v>
       </c>
@@ -4206,7 +5457,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" ht="13">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -4220,7 +5471,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" ht="13">
       <c r="A9" s="1">
         <v>1</v>
       </c>
@@ -4234,7 +5485,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" ht="13">
       <c r="A10" s="1">
         <v>1</v>
       </c>
@@ -4248,7 +5499,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" ht="13">
       <c r="A11" s="1">
         <v>1</v>
       </c>
@@ -4262,7 +5513,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" ht="13">
       <c r="A12" s="1">
         <v>1</v>
       </c>
@@ -4276,7 +5527,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" ht="13">
       <c r="A13" s="1">
         <v>1</v>
       </c>
@@ -4290,7 +5541,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" ht="13">
       <c r="A14" s="1">
         <v>1</v>
       </c>
@@ -4304,7 +5555,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" ht="13">
       <c r="A15" s="1">
         <v>1</v>
       </c>
@@ -4318,7 +5569,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" ht="13">
       <c r="A16" s="1">
         <v>1</v>
       </c>
@@ -4332,7 +5583,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" ht="13">
       <c r="A17" s="1">
         <v>1</v>
       </c>
@@ -12005,6 +13256,3058 @@
       </c>
       <c r="D559" s="1" t="s">
         <v>1248</v>
+      </c>
+    </row>
+    <row r="560" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A560" s="1">
+        <v>10</v>
+      </c>
+      <c r="B560" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C560" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D560" s="12" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="561" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A561" s="1">
+        <v>10</v>
+      </c>
+      <c r="B561" s="12" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C561" s="12" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D561" s="12" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="562" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A562" s="1">
+        <v>10</v>
+      </c>
+      <c r="B562" s="12" t="s">
+        <v>1256</v>
+      </c>
+      <c r="C562" s="12" t="s">
+        <v>1257</v>
+      </c>
+      <c r="D562" s="12" t="s">
+        <v>1258</v>
+      </c>
+    </row>
+    <row r="563" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A563" s="1">
+        <v>10</v>
+      </c>
+      <c r="B563" s="12" t="s">
+        <v>1259</v>
+      </c>
+      <c r="C563" s="12" t="s">
+        <v>1260</v>
+      </c>
+      <c r="D563" s="12" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="564" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A564" s="1">
+        <v>10</v>
+      </c>
+      <c r="B564" s="12" t="s">
+        <v>1262</v>
+      </c>
+      <c r="C564" s="12" t="s">
+        <v>1263</v>
+      </c>
+      <c r="D564" s="12" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="565" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A565" s="1">
+        <v>10</v>
+      </c>
+      <c r="B565" s="12" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C565" s="12" t="s">
+        <v>1266</v>
+      </c>
+      <c r="D565" s="12" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="566" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A566" s="1">
+        <v>10</v>
+      </c>
+      <c r="B566" s="12" t="s">
+        <v>934</v>
+      </c>
+      <c r="C566" s="12" t="s">
+        <v>935</v>
+      </c>
+      <c r="D566" s="12" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="567" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A567" s="1">
+        <v>10</v>
+      </c>
+      <c r="B567" s="12" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C567" s="12" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D567" s="12" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="568" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A568" s="1">
+        <v>10</v>
+      </c>
+      <c r="B568" s="12" t="s">
+        <v>1268</v>
+      </c>
+      <c r="C568" s="12" t="s">
+        <v>1269</v>
+      </c>
+      <c r="D568" s="12" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="569" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A569" s="1">
+        <v>10</v>
+      </c>
+      <c r="B569" s="12" t="s">
+        <v>1271</v>
+      </c>
+      <c r="C569" s="12" t="s">
+        <v>1272</v>
+      </c>
+      <c r="D569" s="12" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="570" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A570" s="1">
+        <v>10</v>
+      </c>
+      <c r="B570" s="12" t="s">
+        <v>1274</v>
+      </c>
+      <c r="C570" s="12" t="s">
+        <v>1275</v>
+      </c>
+      <c r="D570" s="12" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="571" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A571" s="1">
+        <v>10</v>
+      </c>
+      <c r="B571" s="12" t="s">
+        <v>1277</v>
+      </c>
+      <c r="C571" s="12" t="s">
+        <v>1278</v>
+      </c>
+      <c r="D571" s="12" t="s">
+        <v>1279</v>
+      </c>
+    </row>
+    <row r="572" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A572" s="1">
+        <v>10</v>
+      </c>
+      <c r="B572" s="12" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C572" s="12" t="s">
+        <v>1281</v>
+      </c>
+      <c r="D572" s="12" t="s">
+        <v>1282</v>
+      </c>
+    </row>
+    <row r="573" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A573" s="1">
+        <v>10</v>
+      </c>
+      <c r="B573" s="12" t="s">
+        <v>1283</v>
+      </c>
+      <c r="C573" s="12" t="s">
+        <v>1284</v>
+      </c>
+      <c r="D573" s="12" t="s">
+        <v>1285</v>
+      </c>
+    </row>
+    <row r="574" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A574" s="1">
+        <v>10</v>
+      </c>
+      <c r="B574" s="12" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C574" s="12" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D574" s="12" t="s">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="575" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A575" s="1">
+        <v>10</v>
+      </c>
+      <c r="B575" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C575" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D575" s="12" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="576" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A576" s="1">
+        <v>10</v>
+      </c>
+      <c r="B576" s="12" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C576" s="12" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D576" s="12" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="577" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A577" s="1">
+        <v>10</v>
+      </c>
+      <c r="B577" s="12" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C577" s="12" t="s">
+        <v>1288</v>
+      </c>
+      <c r="D577" s="12" t="s">
+        <v>1289</v>
+      </c>
+    </row>
+    <row r="578" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A578" s="1">
+        <v>10</v>
+      </c>
+      <c r="B578" s="12" t="s">
+        <v>1290</v>
+      </c>
+      <c r="C578" s="12" t="s">
+        <v>1291</v>
+      </c>
+      <c r="D578" s="12" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="579" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A579" s="1">
+        <v>10</v>
+      </c>
+      <c r="B579" s="12" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C579" s="12" t="s">
+        <v>1294</v>
+      </c>
+      <c r="D579" s="12" t="s">
+        <v>1295</v>
+      </c>
+    </row>
+    <row r="580" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A580" s="1">
+        <v>10</v>
+      </c>
+      <c r="B580" s="12" t="s">
+        <v>1290</v>
+      </c>
+      <c r="C580" s="12" t="s">
+        <v>1291</v>
+      </c>
+      <c r="D580" s="12" t="s">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="581" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A581" s="1">
+        <v>10</v>
+      </c>
+      <c r="B581" s="12" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C581" s="12" t="s">
+        <v>1298</v>
+      </c>
+      <c r="D581" s="12" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="582" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A582" s="1">
+        <v>10</v>
+      </c>
+      <c r="B582" s="12" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C582" s="12" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D582" s="12" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="583" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A583" s="1">
+        <v>10</v>
+      </c>
+      <c r="B583" s="12" t="s">
+        <v>1300</v>
+      </c>
+      <c r="C583" s="12" t="s">
+        <v>1301</v>
+      </c>
+      <c r="D583" s="12" t="s">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="584" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A584" s="1">
+        <v>10</v>
+      </c>
+      <c r="B584" s="12" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C584" s="12" t="s">
+        <v>1203</v>
+      </c>
+      <c r="D584" s="12" t="s">
+        <v>1204</v>
+      </c>
+    </row>
+    <row r="585" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A585" s="1">
+        <v>10</v>
+      </c>
+      <c r="B585" s="12" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C585" s="12" t="s">
+        <v>1304</v>
+      </c>
+      <c r="D585" s="12" t="s">
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="586" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A586" s="1">
+        <v>10</v>
+      </c>
+      <c r="B586" s="12" t="s">
+        <v>1306</v>
+      </c>
+      <c r="C586" s="12" t="s">
+        <v>1307</v>
+      </c>
+      <c r="D586" s="12" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="587" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A587" s="1">
+        <v>10</v>
+      </c>
+      <c r="B587" s="12" t="s">
+        <v>733</v>
+      </c>
+      <c r="C587" s="12" t="s">
+        <v>734</v>
+      </c>
+      <c r="D587" s="12" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="588" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A588" s="1">
+        <v>10</v>
+      </c>
+      <c r="B588" s="12" t="s">
+        <v>1300</v>
+      </c>
+      <c r="C588" s="12" t="s">
+        <v>1301</v>
+      </c>
+      <c r="D588" s="12" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="589" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A589" s="1">
+        <v>10</v>
+      </c>
+      <c r="B589" s="12" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C589" s="12" t="s">
+        <v>1310</v>
+      </c>
+      <c r="D589" s="12" t="s">
+        <v>1311</v>
+      </c>
+    </row>
+    <row r="590" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A590" s="1">
+        <v>10</v>
+      </c>
+      <c r="B590" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C590" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D590" s="12" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="591" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A591" s="1">
+        <v>10</v>
+      </c>
+      <c r="B591" s="12" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C591" s="12" t="s">
+        <v>1313</v>
+      </c>
+      <c r="D591" s="12" t="s">
+        <v>1314</v>
+      </c>
+    </row>
+    <row r="592" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A592" s="1">
+        <v>10</v>
+      </c>
+      <c r="B592" s="12" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C592" s="12" t="s">
+        <v>1316</v>
+      </c>
+      <c r="D592" s="12" t="s">
+        <v>1317</v>
+      </c>
+    </row>
+    <row r="593" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A593" s="1">
+        <v>10</v>
+      </c>
+      <c r="B593" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="C593" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="D593" s="12" t="s">
+        <v>1318</v>
+      </c>
+    </row>
+    <row r="594" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A594" s="1">
+        <v>10</v>
+      </c>
+      <c r="B594" s="12" t="s">
+        <v>1319</v>
+      </c>
+      <c r="C594" s="12" t="s">
+        <v>1320</v>
+      </c>
+      <c r="D594" s="12" t="s">
+        <v>1321</v>
+      </c>
+    </row>
+    <row r="595" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A595" s="1">
+        <v>10</v>
+      </c>
+      <c r="B595" s="12" t="s">
+        <v>1271</v>
+      </c>
+      <c r="C595" s="12" t="s">
+        <v>1272</v>
+      </c>
+      <c r="D595" s="12" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="596" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A596" s="1">
+        <v>10</v>
+      </c>
+      <c r="B596" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="C596" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="D596" s="12" t="s">
+        <v>1318</v>
+      </c>
+    </row>
+    <row r="597" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A597" s="1">
+        <v>10</v>
+      </c>
+      <c r="B597" s="12" t="s">
+        <v>765</v>
+      </c>
+      <c r="C597" s="12" t="s">
+        <v>766</v>
+      </c>
+      <c r="D597" s="12" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="598" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A598" s="1">
+        <v>10</v>
+      </c>
+      <c r="B598" s="12" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C598" s="12" t="s">
+        <v>1266</v>
+      </c>
+      <c r="D598" s="12" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="599" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A599" s="1">
+        <v>10</v>
+      </c>
+      <c r="B599" s="12" t="s">
+        <v>733</v>
+      </c>
+      <c r="C599" s="12" t="s">
+        <v>734</v>
+      </c>
+      <c r="D599" s="12" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="600" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A600" s="1">
+        <v>10</v>
+      </c>
+      <c r="B600" s="12" t="s">
+        <v>1322</v>
+      </c>
+      <c r="C600" s="12" t="s">
+        <v>1323</v>
+      </c>
+      <c r="D600" s="12" t="s">
+        <v>1324</v>
+      </c>
+    </row>
+    <row r="601" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A601" s="1">
+        <v>10</v>
+      </c>
+      <c r="B601" s="12" t="s">
+        <v>1325</v>
+      </c>
+      <c r="C601" s="12" t="s">
+        <v>1326</v>
+      </c>
+      <c r="D601" s="12" t="s">
+        <v>1327</v>
+      </c>
+    </row>
+    <row r="602" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A602" s="1">
+        <v>10</v>
+      </c>
+      <c r="B602" s="12" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C602" s="12" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D602" s="12" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="603" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A603" s="1">
+        <v>10</v>
+      </c>
+      <c r="B603" s="12" t="s">
+        <v>1328</v>
+      </c>
+      <c r="C603" s="12" t="s">
+        <v>1329</v>
+      </c>
+      <c r="D603" s="12" t="s">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="604" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A604" s="1">
+        <v>10</v>
+      </c>
+      <c r="B604" s="12" t="s">
+        <v>783</v>
+      </c>
+      <c r="C604" s="12" t="s">
+        <v>784</v>
+      </c>
+      <c r="D604" s="12" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="605" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A605" s="1">
+        <v>10</v>
+      </c>
+      <c r="B605" s="12" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C605" s="12" t="s">
+        <v>1332</v>
+      </c>
+      <c r="D605" s="12" t="s">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="606" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A606" s="1">
+        <v>10</v>
+      </c>
+      <c r="B606" s="12" t="s">
+        <v>1334</v>
+      </c>
+      <c r="C606" s="12" t="s">
+        <v>1335</v>
+      </c>
+      <c r="D606" s="12" t="s">
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="607" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A607" s="1">
+        <v>10</v>
+      </c>
+      <c r="B607" s="12" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C607" s="12" t="s">
+        <v>1266</v>
+      </c>
+      <c r="D607" s="12" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="608" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A608" s="1">
+        <v>10</v>
+      </c>
+      <c r="B608" s="12" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C608" s="12" t="s">
+        <v>1141</v>
+      </c>
+      <c r="D608" s="12" t="s">
+        <v>1337</v>
+      </c>
+    </row>
+    <row r="609" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A609" s="1">
+        <v>10</v>
+      </c>
+      <c r="B609" s="12" t="s">
+        <v>801</v>
+      </c>
+      <c r="C609" s="12" t="s">
+        <v>802</v>
+      </c>
+      <c r="D609" s="12" t="s">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="610" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A610" s="1">
+        <v>10</v>
+      </c>
+      <c r="B610" s="12" t="s">
+        <v>810</v>
+      </c>
+      <c r="C610" s="12" t="s">
+        <v>811</v>
+      </c>
+      <c r="D610" s="12" t="s">
+        <v>1339</v>
+      </c>
+    </row>
+    <row r="611" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A611" s="1">
+        <v>10</v>
+      </c>
+      <c r="B611" s="12" t="s">
+        <v>1340</v>
+      </c>
+      <c r="C611" s="12" t="s">
+        <v>1341</v>
+      </c>
+      <c r="D611" s="12" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="612" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A612" s="1">
+        <v>10</v>
+      </c>
+      <c r="B612" s="12" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C612" s="12" t="s">
+        <v>1266</v>
+      </c>
+      <c r="D612" s="12" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="613" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A613" s="1">
+        <v>10</v>
+      </c>
+      <c r="B613" s="12" t="s">
+        <v>1322</v>
+      </c>
+      <c r="C613" s="12" t="s">
+        <v>1323</v>
+      </c>
+      <c r="D613" s="12" t="s">
+        <v>1324</v>
+      </c>
+    </row>
+    <row r="614" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A614" s="1">
+        <v>10</v>
+      </c>
+      <c r="B614" s="12" t="s">
+        <v>1343</v>
+      </c>
+      <c r="C614" s="12" t="s">
+        <v>1344</v>
+      </c>
+      <c r="D614" s="12" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="615" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A615" s="1">
+        <v>10</v>
+      </c>
+      <c r="B615" s="12" t="s">
+        <v>1343</v>
+      </c>
+      <c r="C615" s="12" t="s">
+        <v>1344</v>
+      </c>
+      <c r="D615" s="12" t="s">
+        <v>1346</v>
+      </c>
+    </row>
+    <row r="616" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A616" s="1">
+        <v>10</v>
+      </c>
+      <c r="B616" s="12" t="s">
+        <v>1347</v>
+      </c>
+      <c r="C616" s="12" t="s">
+        <v>1348</v>
+      </c>
+      <c r="D616" s="12" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="617" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A617" s="1">
+        <v>10</v>
+      </c>
+      <c r="B617" s="12" t="s">
+        <v>1349</v>
+      </c>
+      <c r="C617" s="12" t="s">
+        <v>1350</v>
+      </c>
+      <c r="D617" s="12" t="s">
+        <v>1351</v>
+      </c>
+    </row>
+    <row r="618" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A618" s="1">
+        <v>10</v>
+      </c>
+      <c r="B618" s="12" t="s">
+        <v>1352</v>
+      </c>
+      <c r="C618" s="12" t="s">
+        <v>1353</v>
+      </c>
+      <c r="D618" s="12" t="s">
+        <v>1354</v>
+      </c>
+    </row>
+    <row r="619" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A619" s="1">
+        <v>10</v>
+      </c>
+      <c r="B619" s="12" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C619" s="12" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D619" s="12" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="620" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A620" s="1">
+        <v>10</v>
+      </c>
+      <c r="B620" s="12" t="s">
+        <v>1355</v>
+      </c>
+      <c r="C620" s="12" t="s">
+        <v>1356</v>
+      </c>
+      <c r="D620" s="12" t="s">
+        <v>1357</v>
+      </c>
+    </row>
+    <row r="621" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A621" s="1">
+        <v>10</v>
+      </c>
+      <c r="B621" s="12" t="s">
+        <v>1358</v>
+      </c>
+      <c r="C621" s="12" t="s">
+        <v>1359</v>
+      </c>
+      <c r="D621" s="12" t="s">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="622" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A622" s="1">
+        <v>10</v>
+      </c>
+      <c r="B622" s="12" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C622" s="12" t="s">
+        <v>1362</v>
+      </c>
+      <c r="D622" s="12" t="s">
+        <v>1363</v>
+      </c>
+    </row>
+    <row r="623" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A623" s="1">
+        <v>10</v>
+      </c>
+      <c r="B623" s="12" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C623" s="12" t="s">
+        <v>1365</v>
+      </c>
+      <c r="D623" s="12" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="624" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A624" s="1">
+        <v>10</v>
+      </c>
+      <c r="B624" s="12" t="s">
+        <v>1367</v>
+      </c>
+      <c r="C624" s="12" t="s">
+        <v>1368</v>
+      </c>
+      <c r="D624" s="12" t="s">
+        <v>1369</v>
+      </c>
+    </row>
+    <row r="625" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A625" s="1">
+        <v>10</v>
+      </c>
+      <c r="B625" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C625" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D625" s="12" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="626" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A626" s="1">
+        <v>10</v>
+      </c>
+      <c r="B626" s="12" t="s">
+        <v>1370</v>
+      </c>
+      <c r="C626" s="12" t="s">
+        <v>1371</v>
+      </c>
+      <c r="D626" s="12" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="627" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A627" s="1">
+        <v>10</v>
+      </c>
+      <c r="B627" s="12" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C627" s="12" t="s">
+        <v>1374</v>
+      </c>
+      <c r="D627" s="12" t="s">
+        <v>1375</v>
+      </c>
+    </row>
+    <row r="628" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A628" s="1">
+        <v>10</v>
+      </c>
+      <c r="B628" s="12" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C628" s="12" t="s">
+        <v>1377</v>
+      </c>
+      <c r="D628" s="12" t="s">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="629" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A629" s="1">
+        <v>10</v>
+      </c>
+      <c r="B629" s="12" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C629" s="12" t="s">
+        <v>1380</v>
+      </c>
+      <c r="D629" s="12" t="s">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="630" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A630" s="1">
+        <v>10</v>
+      </c>
+      <c r="B630" s="12" t="s">
+        <v>1382</v>
+      </c>
+      <c r="C630" s="12" t="s">
+        <v>1383</v>
+      </c>
+      <c r="D630" s="12" t="s">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="631" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A631" s="1">
+        <v>10</v>
+      </c>
+      <c r="B631" s="12" t="s">
+        <v>1385</v>
+      </c>
+      <c r="C631" s="12" t="s">
+        <v>1386</v>
+      </c>
+      <c r="D631" s="12" t="s">
+        <v>1387</v>
+      </c>
+    </row>
+    <row r="632" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A632" s="1">
+        <v>10</v>
+      </c>
+      <c r="B632" s="12" t="s">
+        <v>1388</v>
+      </c>
+      <c r="C632" s="12" t="s">
+        <v>1389</v>
+      </c>
+      <c r="D632" s="12" t="s">
+        <v>1390</v>
+      </c>
+    </row>
+    <row r="633" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A633" s="1">
+        <v>10</v>
+      </c>
+      <c r="B633" s="12" t="s">
+        <v>1391</v>
+      </c>
+      <c r="C633" s="12" t="s">
+        <v>1392</v>
+      </c>
+      <c r="D633" s="12" t="s">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="634" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A634" s="1">
+        <v>10</v>
+      </c>
+      <c r="B634" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C634" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D634" s="12" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="635" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A635" s="1">
+        <v>10</v>
+      </c>
+      <c r="B635" s="12" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C635" s="12" t="s">
+        <v>1081</v>
+      </c>
+      <c r="D635" s="12" t="s">
+        <v>1394</v>
+      </c>
+    </row>
+    <row r="636" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A636" s="1">
+        <v>10</v>
+      </c>
+      <c r="B636" s="12" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C636" s="12" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D636" s="12" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="637" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A637" s="1">
+        <v>10</v>
+      </c>
+      <c r="B637" s="12" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C637" s="12" t="s">
+        <v>1396</v>
+      </c>
+      <c r="D637" s="12" t="s">
+        <v>1397</v>
+      </c>
+    </row>
+    <row r="638" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A638" s="1">
+        <v>11</v>
+      </c>
+      <c r="B638" s="12" t="s">
+        <v>1398</v>
+      </c>
+      <c r="C638" s="12" t="s">
+        <v>1399</v>
+      </c>
+      <c r="D638" s="12" t="s">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="639" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A639" s="1">
+        <v>11</v>
+      </c>
+      <c r="B639" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C639" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D639" s="12" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="640" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A640" s="1">
+        <v>11</v>
+      </c>
+      <c r="B640" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C640" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D640" s="12" t="s">
+        <v>1401</v>
+      </c>
+    </row>
+    <row r="641" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A641" s="1">
+        <v>11</v>
+      </c>
+      <c r="B641" s="12" t="s">
+        <v>1402</v>
+      </c>
+      <c r="C641" s="12" t="s">
+        <v>1403</v>
+      </c>
+      <c r="D641" s="12" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="642" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A642" s="1">
+        <v>11</v>
+      </c>
+      <c r="B642" s="12" t="s">
+        <v>1405</v>
+      </c>
+      <c r="C642" s="12" t="s">
+        <v>1406</v>
+      </c>
+      <c r="D642" s="12" t="s">
+        <v>1407</v>
+      </c>
+    </row>
+    <row r="643" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A643" s="1">
+        <v>11</v>
+      </c>
+      <c r="B643" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C643" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D643" s="12" t="s">
+        <v>1401</v>
+      </c>
+    </row>
+    <row r="644" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A644" s="1">
+        <v>11</v>
+      </c>
+      <c r="B644" s="12" t="s">
+        <v>1402</v>
+      </c>
+      <c r="C644" s="12" t="s">
+        <v>1403</v>
+      </c>
+      <c r="D644" s="12" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="645" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A645" s="1">
+        <v>11</v>
+      </c>
+      <c r="B645" s="12" t="s">
+        <v>1408</v>
+      </c>
+      <c r="C645" s="12" t="s">
+        <v>1409</v>
+      </c>
+      <c r="D645" s="12" t="s">
+        <v>1410</v>
+      </c>
+    </row>
+    <row r="646" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A646" s="1">
+        <v>11</v>
+      </c>
+      <c r="B646" s="12" t="s">
+        <v>1411</v>
+      </c>
+      <c r="C646" s="12" t="s">
+        <v>1412</v>
+      </c>
+      <c r="D646" s="12" t="s">
+        <v>1413</v>
+      </c>
+    </row>
+    <row r="647" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A647" s="1">
+        <v>11</v>
+      </c>
+      <c r="B647" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C647" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D647" s="12" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="648" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A648" s="1">
+        <v>11</v>
+      </c>
+      <c r="B648" s="12" t="s">
+        <v>1414</v>
+      </c>
+      <c r="C648" s="12" t="s">
+        <v>1415</v>
+      </c>
+      <c r="D648" s="12" t="s">
+        <v>1416</v>
+      </c>
+    </row>
+    <row r="649" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A649" s="1">
+        <v>11</v>
+      </c>
+      <c r="B649" s="12" t="s">
+        <v>1417</v>
+      </c>
+      <c r="C649" s="12" t="s">
+        <v>1418</v>
+      </c>
+      <c r="D649" s="12" t="s">
+        <v>1419</v>
+      </c>
+    </row>
+    <row r="650" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A650" s="1">
+        <v>11</v>
+      </c>
+      <c r="B650" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C650" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D650" s="12" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="651" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A651" s="1">
+        <v>11</v>
+      </c>
+      <c r="B651" s="12" t="s">
+        <v>1414</v>
+      </c>
+      <c r="C651" s="12" t="s">
+        <v>1415</v>
+      </c>
+      <c r="D651" s="12" t="s">
+        <v>1420</v>
+      </c>
+    </row>
+    <row r="652" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A652" s="1">
+        <v>11</v>
+      </c>
+      <c r="B652" s="12" t="s">
+        <v>1421</v>
+      </c>
+      <c r="C652" s="12" t="s">
+        <v>1422</v>
+      </c>
+      <c r="D652" s="12" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="653" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A653" s="1">
+        <v>11</v>
+      </c>
+      <c r="B653" s="12" t="s">
+        <v>724</v>
+      </c>
+      <c r="C653" s="12" t="s">
+        <v>725</v>
+      </c>
+      <c r="D653" s="12" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="654" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A654" s="1">
+        <v>11</v>
+      </c>
+      <c r="B654" s="12" t="s">
+        <v>1424</v>
+      </c>
+      <c r="C654" s="12" t="s">
+        <v>1425</v>
+      </c>
+      <c r="D654" s="12" t="s">
+        <v>1426</v>
+      </c>
+    </row>
+    <row r="655" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A655" s="1">
+        <v>11</v>
+      </c>
+      <c r="B655" s="12" t="s">
+        <v>1427</v>
+      </c>
+      <c r="C655" s="12" t="s">
+        <v>1428</v>
+      </c>
+      <c r="D655" s="12" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="656" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A656" s="1">
+        <v>11</v>
+      </c>
+      <c r="B656" s="12" t="s">
+        <v>621</v>
+      </c>
+      <c r="C656" s="12" t="s">
+        <v>622</v>
+      </c>
+      <c r="D656" s="12" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="657" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A657" s="1">
+        <v>11</v>
+      </c>
+      <c r="B657" s="12" t="s">
+        <v>1402</v>
+      </c>
+      <c r="C657" s="12" t="s">
+        <v>1403</v>
+      </c>
+      <c r="D657" s="12" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="658" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A658" s="1">
+        <v>11</v>
+      </c>
+      <c r="B658" s="12" t="s">
+        <v>1430</v>
+      </c>
+      <c r="C658" s="12" t="s">
+        <v>1431</v>
+      </c>
+      <c r="D658" s="12" t="s">
+        <v>1432</v>
+      </c>
+    </row>
+    <row r="659" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A659" s="1">
+        <v>11</v>
+      </c>
+      <c r="B659" s="12" t="s">
+        <v>1433</v>
+      </c>
+      <c r="C659" s="12" t="s">
+        <v>1434</v>
+      </c>
+      <c r="D659" s="12" t="s">
+        <v>1435</v>
+      </c>
+    </row>
+    <row r="660" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A660" s="1">
+        <v>11</v>
+      </c>
+      <c r="B660" s="12" t="s">
+        <v>1402</v>
+      </c>
+      <c r="C660" s="12" t="s">
+        <v>1403</v>
+      </c>
+      <c r="D660" s="12" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="661" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A661" s="1">
+        <v>11</v>
+      </c>
+      <c r="B661" s="12" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C661" s="12" t="s">
+        <v>1437</v>
+      </c>
+      <c r="D661" s="12" t="s">
+        <v>1438</v>
+      </c>
+    </row>
+    <row r="662" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A662" s="1">
+        <v>11</v>
+      </c>
+      <c r="B662" s="12" t="s">
+        <v>1439</v>
+      </c>
+      <c r="C662" s="12" t="s">
+        <v>1440</v>
+      </c>
+      <c r="D662" s="12" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="663" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A663" s="1">
+        <v>11</v>
+      </c>
+      <c r="B663" s="12" t="s">
+        <v>480</v>
+      </c>
+      <c r="C663" s="12" t="s">
+        <v>481</v>
+      </c>
+      <c r="D663" s="12" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="664" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A664" s="1">
+        <v>11</v>
+      </c>
+      <c r="B664" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="C664" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="D664" s="12" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="665" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A665" s="1">
+        <v>11</v>
+      </c>
+      <c r="B665" s="12" t="s">
+        <v>1442</v>
+      </c>
+      <c r="C665" s="12" t="s">
+        <v>1443</v>
+      </c>
+      <c r="D665" s="12" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="666" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A666" s="1">
+        <v>11</v>
+      </c>
+      <c r="B666" s="12" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C666" s="12" t="s">
+        <v>1446</v>
+      </c>
+      <c r="D666" s="12" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="667" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A667" s="1">
+        <v>11</v>
+      </c>
+      <c r="B667" s="12" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C667" s="12" t="s">
+        <v>1449</v>
+      </c>
+      <c r="D667" s="12" t="s">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="668" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A668" s="1">
+        <v>11</v>
+      </c>
+      <c r="B668" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C668" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D668" s="12" t="s">
+        <v>1401</v>
+      </c>
+    </row>
+    <row r="669" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A669" s="1">
+        <v>11</v>
+      </c>
+      <c r="B669" s="12" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C669" s="12" t="s">
+        <v>1452</v>
+      </c>
+      <c r="D669" s="12" t="s">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="670" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A670" s="1">
+        <v>11</v>
+      </c>
+      <c r="B670" s="12" t="s">
+        <v>1454</v>
+      </c>
+      <c r="C670" s="12" t="s">
+        <v>1455</v>
+      </c>
+      <c r="D670" s="12" t="s">
+        <v>1456</v>
+      </c>
+    </row>
+    <row r="671" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A671" s="1">
+        <v>11</v>
+      </c>
+      <c r="B671" s="12" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C671" s="12" t="s">
+        <v>1458</v>
+      </c>
+      <c r="D671" s="12" t="s">
+        <v>1459</v>
+      </c>
+    </row>
+    <row r="672" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A672" s="1">
+        <v>11</v>
+      </c>
+      <c r="B672" s="12" t="s">
+        <v>1460</v>
+      </c>
+      <c r="C672" s="12" t="s">
+        <v>1460</v>
+      </c>
+      <c r="D672" s="12" t="s">
+        <v>1461</v>
+      </c>
+    </row>
+    <row r="673" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A673" s="1">
+        <v>11</v>
+      </c>
+      <c r="B673" s="12" t="s">
+        <v>1462</v>
+      </c>
+      <c r="C673" s="12" t="s">
+        <v>1463</v>
+      </c>
+      <c r="D673" s="12" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="674" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A674" s="1">
+        <v>11</v>
+      </c>
+      <c r="B674" s="12" t="s">
+        <v>1465</v>
+      </c>
+      <c r="C674" s="12" t="s">
+        <v>1466</v>
+      </c>
+      <c r="D674" s="12" t="s">
+        <v>1467</v>
+      </c>
+    </row>
+    <row r="675" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A675" s="1">
+        <v>11</v>
+      </c>
+      <c r="B675" s="12" t="s">
+        <v>1468</v>
+      </c>
+      <c r="C675" s="12" t="s">
+        <v>1469</v>
+      </c>
+      <c r="D675" s="12" t="s">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="676" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A676" s="1">
+        <v>11</v>
+      </c>
+      <c r="B676" s="12" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C676" s="12" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D676" s="12" t="s">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="677" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A677" s="1">
+        <v>11</v>
+      </c>
+      <c r="B677" s="12" t="s">
+        <v>1474</v>
+      </c>
+      <c r="C677" s="12" t="s">
+        <v>1475</v>
+      </c>
+      <c r="D677" s="12" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="678" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A678" s="1">
+        <v>11</v>
+      </c>
+      <c r="B678" s="12" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C678" s="12" t="s">
+        <v>1452</v>
+      </c>
+      <c r="D678" s="12" t="s">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="679" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A679" s="1">
+        <v>11</v>
+      </c>
+      <c r="B679" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C679" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D679" s="12" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="680" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A680" s="1">
+        <v>11</v>
+      </c>
+      <c r="B680" s="12" t="s">
+        <v>1477</v>
+      </c>
+      <c r="C680" s="12" t="s">
+        <v>1478</v>
+      </c>
+      <c r="D680" s="12" t="s">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="681" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A681" s="1">
+        <v>11</v>
+      </c>
+      <c r="B681" s="12" t="s">
+        <v>1480</v>
+      </c>
+      <c r="C681" s="12" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D681" s="12" t="s">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="682" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A682" s="1">
+        <v>11</v>
+      </c>
+      <c r="B682" s="12" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C682" s="12" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D682" s="12" t="s">
+        <v>1485</v>
+      </c>
+    </row>
+    <row r="683" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A683" s="1">
+        <v>11</v>
+      </c>
+      <c r="B683" s="12" t="s">
+        <v>1486</v>
+      </c>
+      <c r="C683" s="12" t="s">
+        <v>1487</v>
+      </c>
+      <c r="D683" s="12" t="s">
+        <v>1488</v>
+      </c>
+    </row>
+    <row r="684" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A684" s="1">
+        <v>11</v>
+      </c>
+      <c r="B684" s="12" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C684" s="12" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D684" s="12" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="685" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A685" s="1">
+        <v>11</v>
+      </c>
+      <c r="B685" s="12" t="s">
+        <v>486</v>
+      </c>
+      <c r="C685" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D685" s="12" t="s">
+        <v>1490</v>
+      </c>
+    </row>
+    <row r="686" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A686" s="1">
+        <v>11</v>
+      </c>
+      <c r="B686" s="12" t="s">
+        <v>960</v>
+      </c>
+      <c r="C686" s="12" t="s">
+        <v>961</v>
+      </c>
+      <c r="D686" s="12" t="s">
+        <v>1491</v>
+      </c>
+    </row>
+    <row r="687" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A687" s="1">
+        <v>11</v>
+      </c>
+      <c r="B687" s="12" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C687" s="12" t="s">
+        <v>1493</v>
+      </c>
+      <c r="D687" s="12" t="s">
+        <v>1494</v>
+      </c>
+    </row>
+    <row r="688" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A688" s="1">
+        <v>11</v>
+      </c>
+      <c r="B688" s="12" t="s">
+        <v>1495</v>
+      </c>
+      <c r="C688" s="12" t="s">
+        <v>1496</v>
+      </c>
+      <c r="D688" s="12" t="s">
+        <v>1497</v>
+      </c>
+    </row>
+    <row r="689" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A689" s="1">
+        <v>11</v>
+      </c>
+      <c r="B689" s="12" t="s">
+        <v>1498</v>
+      </c>
+      <c r="C689" s="12" t="s">
+        <v>1499</v>
+      </c>
+      <c r="D689" s="12" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="690" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A690" s="1">
+        <v>11</v>
+      </c>
+      <c r="B690" s="12" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C690" s="12" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D690" s="12" t="s">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="691" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A691" s="1">
+        <v>11</v>
+      </c>
+      <c r="B691" s="12" t="s">
+        <v>727</v>
+      </c>
+      <c r="C691" s="12" t="s">
+        <v>728</v>
+      </c>
+      <c r="D691" s="12" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="692" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A692" s="1">
+        <v>11</v>
+      </c>
+      <c r="B692" s="12" t="s">
+        <v>1168</v>
+      </c>
+      <c r="C692" s="12" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D692" s="12" t="s">
+        <v>1242</v>
+      </c>
+    </row>
+    <row r="693" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A693" s="1">
+        <v>11</v>
+      </c>
+      <c r="B693" s="12" t="s">
+        <v>1501</v>
+      </c>
+      <c r="C693" s="12" t="s">
+        <v>1502</v>
+      </c>
+      <c r="D693" s="12" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="694" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A694" s="1">
+        <v>11</v>
+      </c>
+      <c r="B694" s="12" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C694" s="12" t="s">
+        <v>1505</v>
+      </c>
+      <c r="D694" s="12" t="s">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="695" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A695" s="1">
+        <v>11</v>
+      </c>
+      <c r="B695" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C695" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D695" s="12" t="s">
+        <v>1507</v>
+      </c>
+    </row>
+    <row r="696" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A696" s="1">
+        <v>11</v>
+      </c>
+      <c r="B696" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="C696" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="D696" s="12" t="s">
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="697" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A697" s="1">
+        <v>11</v>
+      </c>
+      <c r="B697" s="12" t="s">
+        <v>1462</v>
+      </c>
+      <c r="C697" s="12" t="s">
+        <v>1463</v>
+      </c>
+      <c r="D697" s="12" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="698" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A698" s="1">
+        <v>11</v>
+      </c>
+      <c r="B698" s="12" t="s">
+        <v>1465</v>
+      </c>
+      <c r="C698" s="12" t="s">
+        <v>1466</v>
+      </c>
+      <c r="D698" s="12" t="s">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="699" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A699" s="1">
+        <v>11</v>
+      </c>
+      <c r="B699" s="12" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C699" s="12" t="s">
+        <v>1511</v>
+      </c>
+      <c r="D699" s="12" t="s">
+        <v>1512</v>
+      </c>
+    </row>
+    <row r="700" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A700" s="1">
+        <v>11</v>
+      </c>
+      <c r="B700" s="12" t="s">
+        <v>1513</v>
+      </c>
+      <c r="C700" s="12" t="s">
+        <v>1514</v>
+      </c>
+      <c r="D700" s="12" t="s">
+        <v>1515</v>
+      </c>
+    </row>
+    <row r="701" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A701" s="1">
+        <v>11</v>
+      </c>
+      <c r="B701" s="12" t="s">
+        <v>1516</v>
+      </c>
+      <c r="C701" s="12" t="s">
+        <v>1517</v>
+      </c>
+      <c r="D701" s="12" t="s">
+        <v>1518</v>
+      </c>
+    </row>
+    <row r="702" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A702" s="1">
+        <v>11</v>
+      </c>
+      <c r="B702" s="12" t="s">
+        <v>1519</v>
+      </c>
+      <c r="C702" s="12" t="s">
+        <v>1520</v>
+      </c>
+      <c r="D702" s="12" t="s">
+        <v>1521</v>
+      </c>
+    </row>
+    <row r="703" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A703" s="1">
+        <v>11</v>
+      </c>
+      <c r="B703" s="12" t="s">
+        <v>1522</v>
+      </c>
+      <c r="C703" s="12" t="s">
+        <v>1523</v>
+      </c>
+      <c r="D703" s="12" t="s">
+        <v>1524</v>
+      </c>
+    </row>
+    <row r="704" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A704" s="1">
+        <v>11</v>
+      </c>
+      <c r="B704" s="12" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C704" s="12" t="s">
+        <v>1458</v>
+      </c>
+      <c r="D704" s="12" t="s">
+        <v>1525</v>
+      </c>
+    </row>
+    <row r="705" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A705" s="1">
+        <v>11</v>
+      </c>
+      <c r="B705" s="12" t="s">
+        <v>1460</v>
+      </c>
+      <c r="C705" s="12" t="s">
+        <v>1460</v>
+      </c>
+      <c r="D705" s="12" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="706" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A706" s="1">
+        <v>11</v>
+      </c>
+      <c r="B706" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C706" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D706" s="12" t="s">
+        <v>1401</v>
+      </c>
+    </row>
+    <row r="707" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A707" s="1">
+        <v>11</v>
+      </c>
+      <c r="B707" s="12" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C707" s="12" t="s">
+        <v>1452</v>
+      </c>
+      <c r="D707" s="12" t="s">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="708" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A708" s="1">
+        <v>11</v>
+      </c>
+      <c r="B708" s="12" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C708" s="12" t="s">
+        <v>1528</v>
+      </c>
+      <c r="D708" s="12" t="s">
+        <v>1529</v>
+      </c>
+    </row>
+    <row r="709" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A709" s="1">
+        <v>11</v>
+      </c>
+      <c r="B709" s="12" t="s">
+        <v>1408</v>
+      </c>
+      <c r="C709" s="12" t="s">
+        <v>1409</v>
+      </c>
+      <c r="D709" s="12" t="s">
+        <v>1410</v>
+      </c>
+    </row>
+    <row r="710" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A710" s="1">
+        <v>12</v>
+      </c>
+      <c r="B710" s="12" t="s">
+        <v>1421</v>
+      </c>
+      <c r="C710" s="12" t="s">
+        <v>1422</v>
+      </c>
+      <c r="D710" s="12" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="711" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A711" s="1">
+        <v>12</v>
+      </c>
+      <c r="B711" s="12" t="s">
+        <v>1531</v>
+      </c>
+      <c r="C711" s="12" t="s">
+        <v>1532</v>
+      </c>
+      <c r="D711" s="12" t="s">
+        <v>1533</v>
+      </c>
+    </row>
+    <row r="712" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A712" s="1">
+        <v>12</v>
+      </c>
+      <c r="B712" s="12" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C712" s="12" t="s">
+        <v>1535</v>
+      </c>
+      <c r="D712" s="12" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="713" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A713" s="1">
+        <v>12</v>
+      </c>
+      <c r="B713" s="12" t="s">
+        <v>1421</v>
+      </c>
+      <c r="C713" s="12" t="s">
+        <v>1422</v>
+      </c>
+      <c r="D713" s="12" t="s">
+        <v>1537</v>
+      </c>
+    </row>
+    <row r="714" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A714" s="1">
+        <v>12</v>
+      </c>
+      <c r="B714" s="12" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C714" s="12" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D714" s="12" t="s">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="715" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A715" s="1">
+        <v>12</v>
+      </c>
+      <c r="B715" s="12" t="s">
+        <v>727</v>
+      </c>
+      <c r="C715" s="12" t="s">
+        <v>728</v>
+      </c>
+      <c r="D715" s="12" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="716" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A716" s="1">
+        <v>12</v>
+      </c>
+      <c r="B716" s="12" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C716" s="12" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D716" s="12" t="s">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="717" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A717" s="1">
+        <v>12</v>
+      </c>
+      <c r="B717" s="12" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C717" s="12" t="s">
+        <v>1540</v>
+      </c>
+      <c r="D717" s="12" t="s">
+        <v>1541</v>
+      </c>
+    </row>
+    <row r="718" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A718" s="1">
+        <v>12</v>
+      </c>
+      <c r="B718" s="12" t="s">
+        <v>813</v>
+      </c>
+      <c r="C718" s="12" t="s">
+        <v>814</v>
+      </c>
+      <c r="D718" s="12" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="719" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A719" s="1">
+        <v>12</v>
+      </c>
+      <c r="B719" s="12" t="s">
+        <v>1542</v>
+      </c>
+      <c r="C719" s="12" t="s">
+        <v>1543</v>
+      </c>
+      <c r="D719" s="12" t="s">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="720" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A720" s="1">
+        <v>12</v>
+      </c>
+      <c r="B720" s="12" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C720" s="12" t="s">
+        <v>1535</v>
+      </c>
+      <c r="D720" s="12" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="721" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A721" s="1">
+        <v>12</v>
+      </c>
+      <c r="B721" s="12" t="s">
+        <v>1545</v>
+      </c>
+      <c r="C721" s="12" t="s">
+        <v>1546</v>
+      </c>
+      <c r="D721" s="12" t="s">
+        <v>1547</v>
+      </c>
+    </row>
+    <row r="722" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A722" s="1">
+        <v>12</v>
+      </c>
+      <c r="B722" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C722" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D722" s="12" t="s">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="723" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A723" s="1">
+        <v>12</v>
+      </c>
+      <c r="B723" s="12" t="s">
+        <v>1549</v>
+      </c>
+      <c r="C723" s="12" t="s">
+        <v>1550</v>
+      </c>
+      <c r="D723" s="12" t="s">
+        <v>1551</v>
+      </c>
+    </row>
+    <row r="724" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A724" s="1">
+        <v>12</v>
+      </c>
+      <c r="B724" s="12" t="s">
+        <v>1552</v>
+      </c>
+      <c r="C724" s="12" t="s">
+        <v>1553</v>
+      </c>
+      <c r="D724" s="12" t="s">
+        <v>1554</v>
+      </c>
+    </row>
+    <row r="725" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A725" s="1">
+        <v>12</v>
+      </c>
+      <c r="B725" s="12" t="s">
+        <v>1555</v>
+      </c>
+      <c r="C725" s="12" t="s">
+        <v>1556</v>
+      </c>
+      <c r="D725" s="12" t="s">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="726" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A726" s="1">
+        <v>12</v>
+      </c>
+      <c r="B726" s="12" t="s">
+        <v>1558</v>
+      </c>
+      <c r="C726" s="12" t="s">
+        <v>1559</v>
+      </c>
+      <c r="D726" s="12" t="s">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="727" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A727" s="1">
+        <v>12</v>
+      </c>
+      <c r="B727" s="12" t="s">
+        <v>1561</v>
+      </c>
+      <c r="C727" s="12" t="s">
+        <v>1562</v>
+      </c>
+      <c r="D727" s="12" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="728" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A728" s="1">
+        <v>12</v>
+      </c>
+      <c r="B728" s="12" t="s">
+        <v>1563</v>
+      </c>
+      <c r="C728" s="12" t="s">
+        <v>1564</v>
+      </c>
+      <c r="D728" s="12" t="s">
+        <v>1565</v>
+      </c>
+    </row>
+    <row r="729" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A729" s="1">
+        <v>12</v>
+      </c>
+      <c r="B729" s="12" t="s">
+        <v>1480</v>
+      </c>
+      <c r="C729" s="12" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D729" s="12" t="s">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="730" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A730" s="1">
+        <v>12</v>
+      </c>
+      <c r="B730" s="12" t="s">
+        <v>1566</v>
+      </c>
+      <c r="C730" s="12" t="s">
+        <v>1567</v>
+      </c>
+      <c r="D730" s="12" t="s">
+        <v>1568</v>
+      </c>
+    </row>
+    <row r="731" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A731" s="1">
+        <v>12</v>
+      </c>
+      <c r="B731" s="12" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C731" s="12" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D731" s="12" t="s">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="732" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A732" s="1">
+        <v>12</v>
+      </c>
+      <c r="B732" s="12" t="s">
+        <v>1569</v>
+      </c>
+      <c r="C732" s="12" t="s">
+        <v>1570</v>
+      </c>
+      <c r="D732" s="12" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="733" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A733" s="1">
+        <v>12</v>
+      </c>
+      <c r="B733" s="12" t="s">
+        <v>1571</v>
+      </c>
+      <c r="C733" s="12" t="s">
+        <v>1572</v>
+      </c>
+      <c r="D733" s="12" t="s">
+        <v>1573</v>
+      </c>
+    </row>
+    <row r="734" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A734" s="1">
+        <v>12</v>
+      </c>
+      <c r="B734" s="12" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C734" s="12" t="s">
+        <v>1505</v>
+      </c>
+      <c r="D734" s="12" t="s">
+        <v>1574</v>
+      </c>
+    </row>
+    <row r="735" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A735" s="1">
+        <v>12</v>
+      </c>
+      <c r="B735" s="12" t="s">
+        <v>1575</v>
+      </c>
+      <c r="C735" s="12" t="s">
+        <v>1576</v>
+      </c>
+      <c r="D735" s="12" t="s">
+        <v>1577</v>
+      </c>
+    </row>
+    <row r="736" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A736" s="1">
+        <v>12</v>
+      </c>
+      <c r="B736" s="12" t="s">
+        <v>1578</v>
+      </c>
+      <c r="C736" s="12" t="s">
+        <v>1579</v>
+      </c>
+      <c r="D736" s="12" t="s">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="737" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A737" s="1">
+        <v>12</v>
+      </c>
+      <c r="B737" s="12" t="s">
+        <v>1581</v>
+      </c>
+      <c r="C737" s="12" t="s">
+        <v>1582</v>
+      </c>
+      <c r="D737" s="12" t="s">
+        <v>1583</v>
+      </c>
+    </row>
+    <row r="738" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A738" s="1">
+        <v>12</v>
+      </c>
+      <c r="B738" s="12" t="s">
+        <v>1558</v>
+      </c>
+      <c r="C738" s="12" t="s">
+        <v>1559</v>
+      </c>
+      <c r="D738" s="12" t="s">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="739" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A739" s="1">
+        <v>12</v>
+      </c>
+      <c r="B739" s="12" t="s">
+        <v>1584</v>
+      </c>
+      <c r="C739" s="12" t="s">
+        <v>1585</v>
+      </c>
+      <c r="D739" s="12" t="s">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="740" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A740" s="1">
+        <v>12</v>
+      </c>
+      <c r="B740" s="12" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C740" s="12" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D740" s="12" t="s">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="741" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A741" s="1">
+        <v>12</v>
+      </c>
+      <c r="B741" s="12" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C741" s="12" t="s">
+        <v>1540</v>
+      </c>
+      <c r="D741" s="12" t="s">
+        <v>1541</v>
+      </c>
+    </row>
+    <row r="742" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A742" s="1">
+        <v>12</v>
+      </c>
+      <c r="B742" s="12" t="s">
+        <v>1542</v>
+      </c>
+      <c r="C742" s="12" t="s">
+        <v>1543</v>
+      </c>
+      <c r="D742" s="12" t="s">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="743" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A743" s="1">
+        <v>12</v>
+      </c>
+      <c r="B743" s="12" t="s">
+        <v>1587</v>
+      </c>
+      <c r="C743" s="12" t="s">
+        <v>1588</v>
+      </c>
+      <c r="D743" s="12" t="s">
+        <v>1589</v>
+      </c>
+    </row>
+    <row r="744" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A744" s="1">
+        <v>12</v>
+      </c>
+      <c r="B744" s="12" t="s">
+        <v>1590</v>
+      </c>
+      <c r="C744" s="12" t="s">
+        <v>1591</v>
+      </c>
+      <c r="D744" s="12" t="s">
+        <v>1592</v>
+      </c>
+    </row>
+    <row r="745" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A745" s="1">
+        <v>12</v>
+      </c>
+      <c r="B745" s="12" t="s">
+        <v>1593</v>
+      </c>
+      <c r="C745" s="12" t="s">
+        <v>1593</v>
+      </c>
+      <c r="D745" s="12" t="s">
+        <v>1594</v>
+      </c>
+    </row>
+    <row r="746" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A746" s="1">
+        <v>12</v>
+      </c>
+      <c r="B746" s="12" t="s">
+        <v>1595</v>
+      </c>
+      <c r="C746" s="12" t="s">
+        <v>1596</v>
+      </c>
+      <c r="D746" s="12" t="s">
+        <v>1597</v>
+      </c>
+    </row>
+    <row r="747" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A747" s="1">
+        <v>12</v>
+      </c>
+      <c r="B747" s="12" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C747" s="12" t="s">
+        <v>1599</v>
+      </c>
+      <c r="D747" s="12" t="s">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="748" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A748" s="1">
+        <v>12</v>
+      </c>
+      <c r="B748" s="12" t="s">
+        <v>1601</v>
+      </c>
+      <c r="C748" s="12" t="s">
+        <v>1602</v>
+      </c>
+      <c r="D748" s="12" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="749" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A749" s="1">
+        <v>12</v>
+      </c>
+      <c r="B749" s="12" t="s">
+        <v>1604</v>
+      </c>
+      <c r="C749" s="12" t="s">
+        <v>1605</v>
+      </c>
+      <c r="D749" s="12" t="s">
+        <v>1606</v>
+      </c>
+    </row>
+    <row r="750" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A750" s="1">
+        <v>12</v>
+      </c>
+      <c r="B750" s="12" t="s">
+        <v>1607</v>
+      </c>
+      <c r="C750" s="12" t="s">
+        <v>1608</v>
+      </c>
+      <c r="D750" s="12" t="s">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="751" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A751" s="1">
+        <v>12</v>
+      </c>
+      <c r="B751" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C751" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D751" s="12" t="s">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="752" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A752" s="1">
+        <v>12</v>
+      </c>
+      <c r="B752" s="12" t="s">
+        <v>1609</v>
+      </c>
+      <c r="C752" s="12" t="s">
+        <v>1609</v>
+      </c>
+      <c r="D752" s="12" t="s">
+        <v>1610</v>
+      </c>
+    </row>
+    <row r="753" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A753" s="1">
+        <v>12</v>
+      </c>
+      <c r="B753" s="12" t="s">
+        <v>1611</v>
+      </c>
+      <c r="C753" s="12" t="s">
+        <v>1612</v>
+      </c>
+      <c r="D753" s="12" t="s">
+        <v>1613</v>
+      </c>
+    </row>
+    <row r="754" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A754" s="1">
+        <v>12</v>
+      </c>
+      <c r="B754" s="12" t="s">
+        <v>1614</v>
+      </c>
+      <c r="C754" s="12" t="s">
+        <v>1615</v>
+      </c>
+      <c r="D754" s="12" t="s">
+        <v>1616</v>
+      </c>
+    </row>
+    <row r="755" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A755" s="1">
+        <v>12</v>
+      </c>
+      <c r="B755" s="12" t="s">
+        <v>1617</v>
+      </c>
+      <c r="C755" s="12" t="s">
+        <v>1618</v>
+      </c>
+      <c r="D755" s="12" t="s">
+        <v>1619</v>
+      </c>
+    </row>
+    <row r="756" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A756" s="1">
+        <v>12</v>
+      </c>
+      <c r="B756" s="12" t="s">
+        <v>1402</v>
+      </c>
+      <c r="C756" s="12" t="s">
+        <v>1403</v>
+      </c>
+      <c r="D756" s="12" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="757" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A757" s="1">
+        <v>12</v>
+      </c>
+      <c r="B757" s="12" t="s">
+        <v>1620</v>
+      </c>
+      <c r="C757" s="12" t="s">
+        <v>1621</v>
+      </c>
+      <c r="D757" s="12" t="s">
+        <v>1622</v>
+      </c>
+    </row>
+    <row r="758" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A758" s="1">
+        <v>12</v>
+      </c>
+      <c r="B758" s="12" t="s">
+        <v>1623</v>
+      </c>
+      <c r="C758" s="12" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D758" s="12" t="s">
+        <v>1625</v>
+      </c>
+    </row>
+    <row r="759" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A759" s="1">
+        <v>12</v>
+      </c>
+      <c r="B759" s="12" t="s">
+        <v>1626</v>
+      </c>
+      <c r="C759" s="12" t="s">
+        <v>1627</v>
+      </c>
+      <c r="D759" s="12" t="s">
+        <v>1628</v>
+      </c>
+    </row>
+    <row r="760" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A760" s="1">
+        <v>12</v>
+      </c>
+      <c r="B760" s="12" t="s">
+        <v>1474</v>
+      </c>
+      <c r="C760" s="12" t="s">
+        <v>1475</v>
+      </c>
+      <c r="D760" s="12" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="761" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A761" s="1">
+        <v>12</v>
+      </c>
+      <c r="B761" s="12" t="s">
+        <v>1629</v>
+      </c>
+      <c r="C761" s="12" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D761" s="12" t="s">
+        <v>1631</v>
+      </c>
+    </row>
+    <row r="762" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A762" s="1">
+        <v>12</v>
+      </c>
+      <c r="B762" s="12" t="s">
+        <v>1632</v>
+      </c>
+      <c r="C762" s="12" t="s">
+        <v>1633</v>
+      </c>
+      <c r="D762" s="12" t="s">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="763" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A763" s="1">
+        <v>12</v>
+      </c>
+      <c r="B763" s="12" t="s">
+        <v>1635</v>
+      </c>
+      <c r="C763" s="12" t="s">
+        <v>1636</v>
+      </c>
+      <c r="D763" s="12" t="s">
+        <v>1637</v>
+      </c>
+    </row>
+    <row r="764" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A764" s="1">
+        <v>12</v>
+      </c>
+      <c r="B764" s="12" t="s">
+        <v>1638</v>
+      </c>
+      <c r="C764" s="12" t="s">
+        <v>1639</v>
+      </c>
+      <c r="D764" s="12" t="s">
+        <v>1640</v>
+      </c>
+    </row>
+    <row r="765" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A765" s="1">
+        <v>12</v>
+      </c>
+      <c r="B765" s="12" t="s">
+        <v>1635</v>
+      </c>
+      <c r="C765" s="12" t="s">
+        <v>1636</v>
+      </c>
+      <c r="D765" s="12" t="s">
+        <v>1641</v>
+      </c>
+    </row>
+    <row r="766" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A766" s="1">
+        <v>12</v>
+      </c>
+      <c r="B766" s="12" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C766" s="12" t="s">
+        <v>1446</v>
+      </c>
+      <c r="D766" s="12" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="767" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A767" s="1">
+        <v>12</v>
+      </c>
+      <c r="B767" s="12" t="s">
+        <v>1642</v>
+      </c>
+      <c r="C767" s="12" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D767" s="12" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="768" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A768" s="1">
+        <v>12</v>
+      </c>
+      <c r="B768" s="12" t="s">
+        <v>1262</v>
+      </c>
+      <c r="C768" s="12" t="s">
+        <v>1263</v>
+      </c>
+      <c r="D768" s="12" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="769" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A769" s="1">
+        <v>12</v>
+      </c>
+      <c r="B769" s="12" t="s">
+        <v>1645</v>
+      </c>
+      <c r="C769" s="12" t="s">
+        <v>1646</v>
+      </c>
+      <c r="D769" s="12" t="s">
+        <v>1647</v>
+      </c>
+    </row>
+    <row r="770" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A770" s="1">
+        <v>12</v>
+      </c>
+      <c r="B770" s="12" t="s">
+        <v>1611</v>
+      </c>
+      <c r="C770" s="12" t="s">
+        <v>1612</v>
+      </c>
+      <c r="D770" s="12" t="s">
+        <v>1613</v>
+      </c>
+    </row>
+    <row r="771" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A771" s="1">
+        <v>12</v>
+      </c>
+      <c r="B771" s="12" t="s">
+        <v>1648</v>
+      </c>
+      <c r="C771" s="12" t="s">
+        <v>1649</v>
+      </c>
+      <c r="D771" s="12" t="s">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="772" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A772" s="1">
+        <v>12</v>
+      </c>
+      <c r="B772" s="12" t="s">
+        <v>1651</v>
+      </c>
+      <c r="C772" s="12" t="s">
+        <v>1652</v>
+      </c>
+      <c r="D772" s="12" t="s">
+        <v>1653</v>
+      </c>
+    </row>
+    <row r="773" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A773" s="1">
+        <v>12</v>
+      </c>
+      <c r="B773" s="12" t="s">
+        <v>1654</v>
+      </c>
+      <c r="C773" s="12" t="s">
+        <v>1655</v>
+      </c>
+      <c r="D773" s="12" t="s">
+        <v>1656</v>
+      </c>
+    </row>
+    <row r="774" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A774" s="1">
+        <v>12</v>
+      </c>
+      <c r="B774" s="12" t="s">
+        <v>1657</v>
+      </c>
+      <c r="C774" s="12" t="s">
+        <v>1658</v>
+      </c>
+      <c r="D774" s="12" t="s">
+        <v>1659</v>
+      </c>
+    </row>
+    <row r="775" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A775" s="1">
+        <v>12</v>
+      </c>
+      <c r="B775" s="12" t="s">
+        <v>1660</v>
+      </c>
+      <c r="C775" s="12" t="s">
+        <v>1661</v>
+      </c>
+      <c r="D775" s="12" t="s">
+        <v>1662</v>
+      </c>
+    </row>
+    <row r="776" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A776" s="1">
+        <v>12</v>
+      </c>
+      <c r="B776" s="12" t="s">
+        <v>1663</v>
+      </c>
+      <c r="C776" s="12" t="s">
+        <v>1664</v>
+      </c>
+      <c r="D776" s="12" t="s">
+        <v>1665</v>
+      </c>
+    </row>
+    <row r="777" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A777" s="1">
+        <v>12</v>
+      </c>
+      <c r="B777" s="12" t="s">
+        <v>1666</v>
+      </c>
+      <c r="C777" s="12" t="s">
+        <v>1667</v>
+      </c>
+      <c r="D777" s="12" t="s">
+        <v>1668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tambah kotoba sampe hal 21
</commit_message>
<xml_diff>
--- a/public/kotoba_mokuzai.xlsx
+++ b/public/kotoba_mokuzai.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\mokuzai_flashcard\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DEB2AA-4956-4E1A-8868-BD6790E5E2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{263A5C2A-6175-41CD-A980-F96E49F943F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3355" uniqueCount="2188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4186" uniqueCount="2517">
   <si>
     <t>第１章</t>
   </si>
@@ -6584,6 +6584,993 @@
   </si>
   <si>
     <t>かくざい</t>
+  </si>
+  <si>
+    <t>kayu laminasi (glulam)</t>
+  </si>
+  <si>
+    <t>kayu laminasi</t>
+  </si>
+  <si>
+    <t>乾燥</t>
+  </si>
+  <si>
+    <t>かんそう</t>
+  </si>
+  <si>
+    <t>pengeringan; kering</t>
+  </si>
+  <si>
+    <t>ラミナ</t>
+  </si>
+  <si>
+    <t>lamina (lembaran kayu penyusun glulam)</t>
+  </si>
+  <si>
+    <t>ukuran, dimensi</t>
+  </si>
+  <si>
+    <t>精度</t>
+  </si>
+  <si>
+    <t>せいど</t>
+  </si>
+  <si>
+    <t>tingkat ketelitian, akurasi</t>
+  </si>
+  <si>
+    <t>安定性</t>
+  </si>
+  <si>
+    <t>あんていせい</t>
+  </si>
+  <si>
+    <t>kestabilan</t>
+  </si>
+  <si>
+    <t>特徴</t>
+  </si>
+  <si>
+    <t>とくちょう</t>
+  </si>
+  <si>
+    <t>ciri khas, karakteristik</t>
+  </si>
+  <si>
+    <t>mata kayu (knot)</t>
+  </si>
+  <si>
+    <t>取り除く</t>
+  </si>
+  <si>
+    <t>とりのぞく</t>
+  </si>
+  <si>
+    <t>menghilangkan</t>
+  </si>
+  <si>
+    <t>強度性能</t>
+  </si>
+  <si>
+    <t>きょうどせいのう</t>
+  </si>
+  <si>
+    <t>performa kekuatan</t>
+  </si>
+  <si>
+    <t>sedikit</t>
+  </si>
+  <si>
+    <t>安定する</t>
+  </si>
+  <si>
+    <t>あんていする</t>
+  </si>
+  <si>
+    <t>stabil</t>
+  </si>
+  <si>
+    <t>karakteristik</t>
+  </si>
+  <si>
+    <t>幅</t>
+  </si>
+  <si>
+    <t>はば</t>
+  </si>
+  <si>
+    <t>lebar</t>
+  </si>
+  <si>
+    <t>自由</t>
+  </si>
+  <si>
+    <t>じゆう</t>
+  </si>
+  <si>
+    <t>bebas</t>
+  </si>
+  <si>
+    <t>接着</t>
+  </si>
+  <si>
+    <t>せっちゃく</t>
+  </si>
+  <si>
+    <t>perekatan, pengeleman</t>
+  </si>
+  <si>
+    <t>サイズ</t>
+  </si>
+  <si>
+    <t>ukuran (size)</t>
+  </si>
+  <si>
+    <t>自由度</t>
+  </si>
+  <si>
+    <t>じゆうど</t>
+  </si>
+  <si>
+    <t>tingkat fleksibilitas</t>
+  </si>
+  <si>
+    <t>曲がる</t>
+  </si>
+  <si>
+    <t>まがる</t>
+  </si>
+  <si>
+    <t>melengkung</t>
+  </si>
+  <si>
+    <t>用語解説</t>
+  </si>
+  <si>
+    <t>ようごかいせつ</t>
+  </si>
+  <si>
+    <t>penjelasan istilah</t>
+  </si>
+  <si>
+    <t>構成する</t>
+  </si>
+  <si>
+    <t>こうせいする</t>
+  </si>
+  <si>
+    <t>menyusun, membentuk</t>
+  </si>
+  <si>
+    <t>挽板</t>
+  </si>
+  <si>
+    <t>papan hasil gergajian (lamina)</t>
+  </si>
+  <si>
+    <t>板材</t>
+  </si>
+  <si>
+    <t>いたざい</t>
+  </si>
+  <si>
+    <t>papan kayu</t>
+  </si>
+  <si>
+    <t>balok persegi kecil</t>
+  </si>
+  <si>
+    <t>arah lebar</t>
+  </si>
+  <si>
+    <t>perekatan</t>
+  </si>
+  <si>
+    <t>kayu laminasi struktural (structural glulam)</t>
+  </si>
+  <si>
+    <t>kayu laminasi struktural</t>
+  </si>
+  <si>
+    <t>balok</t>
+  </si>
+  <si>
+    <t>balok dasar, fondasi</t>
+  </si>
+  <si>
+    <t>耐力部材</t>
+  </si>
+  <si>
+    <t>たいりょくぶざい</t>
+  </si>
+  <si>
+    <t>komponen penahan beban</t>
+  </si>
+  <si>
+    <t>penampang</t>
+  </si>
+  <si>
+    <t>大断面</t>
+  </si>
+  <si>
+    <t>だいだんめん</t>
+  </si>
+  <si>
+    <t>penampang besar</t>
+  </si>
+  <si>
+    <t>断面積</t>
+  </si>
+  <si>
+    <t>だんめんせき</t>
+  </si>
+  <si>
+    <t>luas penampang</t>
+  </si>
+  <si>
+    <t>中断面</t>
+  </si>
+  <si>
+    <t>ちゅうだんめん</t>
+  </si>
+  <si>
+    <t>penampang sedang</t>
+  </si>
+  <si>
+    <t>又は</t>
+  </si>
+  <si>
+    <t>または</t>
+  </si>
+  <si>
+    <t>atau</t>
+  </si>
+  <si>
+    <t>中断面集成材</t>
+  </si>
+  <si>
+    <t>ちゅうだんめんしゅうせいざい</t>
+  </si>
+  <si>
+    <t>glulam penampang sedang</t>
+  </si>
+  <si>
+    <t>桁</t>
+  </si>
+  <si>
+    <t>けた</t>
+  </si>
+  <si>
+    <t>girder/balok memanjang</t>
+  </si>
+  <si>
+    <t>小断面集成材</t>
+  </si>
+  <si>
+    <t>しょうだんめんしゅうせいざい</t>
+  </si>
+  <si>
+    <t>glulam penampang kecil</t>
+  </si>
+  <si>
+    <t>balok dasar</t>
+  </si>
+  <si>
+    <t>小・中断面集成材</t>
+  </si>
+  <si>
+    <t>しょう・ちゅうだんめんしゅうせいざい</t>
+  </si>
+  <si>
+    <t>glulam penampang kecil dan sedang</t>
+  </si>
+  <si>
+    <t>住宅</t>
+  </si>
+  <si>
+    <t>じゅうたく</t>
+  </si>
+  <si>
+    <t>rumah tinggal</t>
+  </si>
+  <si>
+    <t>大断面集成材</t>
+  </si>
+  <si>
+    <t>だいだんめんしゅうせいざい</t>
+  </si>
+  <si>
+    <t>glulam penampang besar</t>
+  </si>
+  <si>
+    <t>体育館</t>
+  </si>
+  <si>
+    <t>たいいくかん</t>
+  </si>
+  <si>
+    <t>gedung olahraga</t>
+  </si>
+  <si>
+    <t>商業施設</t>
+  </si>
+  <si>
+    <t>しょうぎょうしせつ</t>
+  </si>
+  <si>
+    <t>fasilitas komersial</t>
+  </si>
+  <si>
+    <t>非住宅木造建築物</t>
+  </si>
+  <si>
+    <t>ひじゅうたくもくぞうけんちくぶつ</t>
+  </si>
+  <si>
+    <t>bangunan kayu non-perumahan</t>
+  </si>
+  <si>
+    <t>決める</t>
+  </si>
+  <si>
+    <t>きめる</t>
+  </si>
+  <si>
+    <t>menetapkan</t>
+  </si>
+  <si>
+    <t>強度等級</t>
+  </si>
+  <si>
+    <t>きょうどとうきゅう</t>
+  </si>
+  <si>
+    <t>kelas kekuatan</t>
+  </si>
+  <si>
+    <t>表示</t>
+  </si>
+  <si>
+    <t>ひょうじ</t>
+  </si>
+  <si>
+    <t>penandaan, tampilan</t>
+  </si>
+  <si>
+    <t>曲げヤング係数</t>
+  </si>
+  <si>
+    <t>まげヤングけいすう</t>
+  </si>
+  <si>
+    <t>modulus Young untuk pembengkokan</t>
+  </si>
+  <si>
+    <t>menunjukkan</t>
+  </si>
+  <si>
+    <t>数字</t>
+  </si>
+  <si>
+    <t>すうじ</t>
+  </si>
+  <si>
+    <t>angka</t>
+  </si>
+  <si>
+    <t>美観</t>
+  </si>
+  <si>
+    <t>びかん</t>
+  </si>
+  <si>
+    <t>keindahan tampilan</t>
+  </si>
+  <si>
+    <t>目的</t>
+  </si>
+  <si>
+    <t>もくてき</t>
+  </si>
+  <si>
+    <t>tujuan</t>
+  </si>
+  <si>
+    <t>表面</t>
+  </si>
+  <si>
+    <t>ひょうめん</t>
+  </si>
+  <si>
+    <t>化粧薄板</t>
+  </si>
+  <si>
+    <t>けしょううすいた</t>
+  </si>
+  <si>
+    <t>veneer dekoratif</t>
+  </si>
+  <si>
+    <t>貼り付ける</t>
+  </si>
+  <si>
+    <t>はりつける</t>
+  </si>
+  <si>
+    <t>menempelkan</t>
+  </si>
+  <si>
+    <t>化粧ばり構造用集成柱</t>
+  </si>
+  <si>
+    <t>けしょうばりこうぞうようしゅうせいばしら</t>
+  </si>
+  <si>
+    <t>kolom glulam struktural berlapis veneer dekoratif</t>
+  </si>
+  <si>
+    <t>和室</t>
+  </si>
+  <si>
+    <t>わしつ</t>
+  </si>
+  <si>
+    <t>ruang bergaya Jepang</t>
+  </si>
+  <si>
+    <t>造作用集成材</t>
+  </si>
+  <si>
+    <t>ぞうさくようしゅうせいざい</t>
+  </si>
+  <si>
+    <t>kayu laminasi untuk keperluan interior/finishing</t>
+  </si>
+  <si>
+    <t>kayu laminasi untuk keperluan interior</t>
+  </si>
+  <si>
+    <t>keindahan tampilan, estetika</t>
+  </si>
+  <si>
+    <t>備える</t>
+  </si>
+  <si>
+    <t>そなえる</t>
+  </si>
+  <si>
+    <t>memiliki, dilengkapi dengan</t>
+  </si>
+  <si>
+    <t>内部造作</t>
+  </si>
+  <si>
+    <t>ないぶぞうさく</t>
+  </si>
+  <si>
+    <t>pekerjaan interior/finishing bagian dalam bangunan</t>
+  </si>
+  <si>
+    <t>化粧ばり造作用集成材</t>
+  </si>
+  <si>
+    <t>けしょうばりぞうさくようしゅうせいざい</t>
+  </si>
+  <si>
+    <t>kayu laminasi interior yang dilapisi veneer dekoratif</t>
+  </si>
+  <si>
+    <t>kayu laminasi interior berlapis veneer dekoratif</t>
+  </si>
+  <si>
+    <t>溝切り</t>
+  </si>
+  <si>
+    <t>みぞきり</t>
+  </si>
+  <si>
+    <t>pembuatan alur/grooving</t>
+  </si>
+  <si>
+    <t>飾り</t>
+  </si>
+  <si>
+    <t>かざり</t>
+  </si>
+  <si>
+    <t>hiasan, dekorasi</t>
+  </si>
+  <si>
+    <t>施す</t>
+  </si>
+  <si>
+    <t>ほどこす</t>
+  </si>
+  <si>
+    <t>memberikan, menerapkan, membuat (dekorasi/perlakuan)</t>
+  </si>
+  <si>
+    <t>kayu lapis (plywood)</t>
+  </si>
+  <si>
+    <t>kayu lapis</t>
+  </si>
+  <si>
+    <t>広い</t>
+  </si>
+  <si>
+    <t>ひろい</t>
+  </si>
+  <si>
+    <t>luas</t>
+  </si>
+  <si>
+    <t>面積</t>
+  </si>
+  <si>
+    <t>めんせき</t>
+  </si>
+  <si>
+    <t>luas area</t>
+  </si>
+  <si>
+    <t>伸び縮み</t>
+  </si>
+  <si>
+    <t>のびちぢみ</t>
+  </si>
+  <si>
+    <t>pemuaian dan penyusutan</t>
+  </si>
+  <si>
+    <t>寸法安定性</t>
+  </si>
+  <si>
+    <t>すんぽうあんていせい</t>
+  </si>
+  <si>
+    <t>kestabilan dimensi</t>
+  </si>
+  <si>
+    <t>特長</t>
+  </si>
+  <si>
+    <t>karakteristik, keunggulan</t>
+  </si>
+  <si>
+    <t>建物</t>
+  </si>
+  <si>
+    <t>たてもの</t>
+  </si>
+  <si>
+    <t>関する</t>
+  </si>
+  <si>
+    <t>かんする</t>
+  </si>
+  <si>
+    <t>berkaitan dengan</t>
+  </si>
+  <si>
+    <t>楽器</t>
+  </si>
+  <si>
+    <t>がっき</t>
+  </si>
+  <si>
+    <t>alat musik</t>
+  </si>
+  <si>
+    <t>運動用具</t>
+  </si>
+  <si>
+    <t>うんどうようぐ</t>
+  </si>
+  <si>
+    <t>peralatan olahraga</t>
+  </si>
+  <si>
+    <t>kehidupan sehari-hari</t>
+  </si>
+  <si>
+    <t>鉄道</t>
+  </si>
+  <si>
+    <t>てつどう</t>
+  </si>
+  <si>
+    <t>kereta api</t>
+  </si>
+  <si>
+    <t>車両</t>
+  </si>
+  <si>
+    <t>しゃりょう</t>
+  </si>
+  <si>
+    <t>kendaraan/gerbong</t>
+  </si>
+  <si>
+    <t>荷台</t>
+  </si>
+  <si>
+    <t>にだい</t>
+  </si>
+  <si>
+    <t>bak kendaraan (truk)</t>
+  </si>
+  <si>
+    <t>乗物</t>
+  </si>
+  <si>
+    <t>のりもの</t>
+  </si>
+  <si>
+    <t>kendaraan</t>
+  </si>
+  <si>
+    <t>sangat beragam, luas</t>
+  </si>
+  <si>
+    <t>コンクリート型枠用合板</t>
+  </si>
+  <si>
+    <t>コンクリートかたわくようごうはん</t>
+  </si>
+  <si>
+    <t>plywood untuk bekisting beton</t>
+  </si>
+  <si>
+    <t>定める</t>
+  </si>
+  <si>
+    <t>さだめる</t>
+  </si>
+  <si>
+    <t>木工製品</t>
+  </si>
+  <si>
+    <t>もっこうせいひん</t>
+  </si>
+  <si>
+    <t>produk pertukangan kayu</t>
+  </si>
+  <si>
+    <t>広く</t>
+  </si>
+  <si>
+    <t>ひろく</t>
+  </si>
+  <si>
+    <t>secara luas</t>
+  </si>
+  <si>
+    <t>plywood</t>
+  </si>
+  <si>
+    <t>主</t>
+  </si>
+  <si>
+    <t>おも</t>
+  </si>
+  <si>
+    <t>原料</t>
+  </si>
+  <si>
+    <t>げんりょう</t>
+  </si>
+  <si>
+    <t>tipis</t>
+  </si>
+  <si>
+    <t>薄物合板</t>
+  </si>
+  <si>
+    <t>うすものごうはん</t>
+  </si>
+  <si>
+    <t>plywood tipis</t>
+  </si>
+  <si>
+    <t>plywood bekisting beton</t>
+  </si>
+  <si>
+    <t>tertentu, tetap</t>
+  </si>
+  <si>
+    <t>強度</t>
+  </si>
+  <si>
+    <t>きょうど</t>
+  </si>
+  <si>
+    <t>耐水性能</t>
+  </si>
+  <si>
+    <t>たいすいせいのう</t>
+  </si>
+  <si>
+    <t>ketahanan terhadap air</t>
+  </si>
+  <si>
+    <t>流し込む</t>
+  </si>
+  <si>
+    <t>ながしこむ</t>
+  </si>
+  <si>
+    <t>menuangkan</t>
+  </si>
+  <si>
+    <t>成形</t>
+  </si>
+  <si>
+    <t>せいけい</t>
+  </si>
+  <si>
+    <t>pembentukan, pencetakan</t>
+  </si>
+  <si>
+    <t>型枠</t>
+  </si>
+  <si>
+    <t>かたわく</t>
+  </si>
+  <si>
+    <t>cetakan/bekisting</t>
+  </si>
+  <si>
+    <t>建設</t>
+  </si>
+  <si>
+    <t>けんせつ</t>
+  </si>
+  <si>
+    <t>konstruksi</t>
+  </si>
+  <si>
+    <t>土木工事</t>
+  </si>
+  <si>
+    <t>どぼくこうじ</t>
+  </si>
+  <si>
+    <t>pekerjaan sipil</t>
+  </si>
+  <si>
+    <t>現場</t>
+  </si>
+  <si>
+    <t>げんば</t>
+  </si>
+  <si>
+    <t>lokasi kerja, lapangan</t>
+  </si>
+  <si>
+    <t>打設</t>
+  </si>
+  <si>
+    <t>だせつ</t>
+  </si>
+  <si>
+    <t>pengecoran beton</t>
+  </si>
+  <si>
+    <t>後</t>
+  </si>
+  <si>
+    <t>ご</t>
+  </si>
+  <si>
+    <t>setelah</t>
+  </si>
+  <si>
+    <t>滑らか</t>
+  </si>
+  <si>
+    <t>なめらか</t>
+  </si>
+  <si>
+    <t>halus, rata</t>
+  </si>
+  <si>
+    <t>付きにくい</t>
+  </si>
+  <si>
+    <t>つきにくい</t>
+  </si>
+  <si>
+    <t>sulit menempel</t>
+  </si>
+  <si>
+    <t>塗装</t>
+  </si>
+  <si>
+    <t>とそう</t>
+  </si>
+  <si>
+    <t>pelapisan cat, coating</t>
+  </si>
+  <si>
+    <t>仕上げ加工</t>
+  </si>
+  <si>
+    <t>しあげかこう</t>
+  </si>
+  <si>
+    <t>proses finishing</t>
+  </si>
+  <si>
+    <t>構造耐力上</t>
+  </si>
+  <si>
+    <t>こうぞうたいりょくじょう</t>
+  </si>
+  <si>
+    <t>dari segi kekuatan struktur</t>
+  </si>
+  <si>
+    <t>bagian, lokasi</t>
+  </si>
+  <si>
+    <t>下地材</t>
+  </si>
+  <si>
+    <t>したじざい</t>
+  </si>
+  <si>
+    <t>bahan dasar/lapisan dasar</t>
+  </si>
+  <si>
+    <t>国産針葉樹</t>
+  </si>
+  <si>
+    <t>こくさんしんようじゅ</t>
+  </si>
+  <si>
+    <t>pohon konifer produksi dalam negeri</t>
+  </si>
+  <si>
+    <t>普及</t>
+  </si>
+  <si>
+    <t>ふきゅう</t>
+  </si>
+  <si>
+    <t>penyebaran, penggunaan luas</t>
+  </si>
+  <si>
+    <t>khususnya</t>
+  </si>
+  <si>
+    <t>厚物構造用合板</t>
+  </si>
+  <si>
+    <t>あつものこうぞうようごうはん</t>
+  </si>
+  <si>
+    <t>plywood struktural tebal</t>
+  </si>
+  <si>
+    <t>balok penyangga lantai (floor joist)</t>
+  </si>
+  <si>
+    <t>省略</t>
+  </si>
+  <si>
+    <t>しょうりゃく</t>
+  </si>
+  <si>
+    <t>penghilangan, penyederhanaan</t>
+  </si>
+  <si>
+    <t>進む</t>
+  </si>
+  <si>
+    <t>すすむ</t>
+  </si>
+  <si>
+    <t>berkembang, maju</t>
+  </si>
+  <si>
+    <t>強度試験</t>
+  </si>
+  <si>
+    <t>きょうどしけん</t>
+  </si>
+  <si>
+    <t>uji kekuatan</t>
+  </si>
+  <si>
+    <t>kelas/tingkat</t>
+  </si>
+  <si>
+    <t>接着性能</t>
+  </si>
+  <si>
+    <t>せっちゃくせいのう</t>
+  </si>
+  <si>
+    <t>performa daya rekat</t>
+  </si>
+  <si>
+    <t>特類</t>
+  </si>
+  <si>
+    <t>とくるい</t>
+  </si>
+  <si>
+    <t>kelas khusus</t>
+  </si>
+  <si>
+    <t>kategori/kelas</t>
+  </si>
+  <si>
+    <t>secara umum</t>
+  </si>
+  <si>
+    <t>bahan lapisan dasar</t>
+  </si>
+  <si>
+    <t>kelas</t>
+  </si>
+  <si>
+    <t>gambar, ilustrasi</t>
+  </si>
+  <si>
+    <t>使用例</t>
+  </si>
+  <si>
+    <t>しようれい</t>
+  </si>
+  <si>
+    <t>contoh penggunaan</t>
+  </si>
+  <si>
+    <t>写真</t>
+  </si>
+  <si>
+    <t>しゃしん</t>
+  </si>
+  <si>
+    <t>foto</t>
+  </si>
+  <si>
+    <t>工業</t>
+  </si>
+  <si>
+    <t>こうぎょう</t>
+  </si>
+  <si>
+    <t>industri</t>
+  </si>
+  <si>
+    <t>組合</t>
+  </si>
+  <si>
+    <t>くみあい</t>
+  </si>
+  <si>
+    <t>asosiasi, serikat</t>
+  </si>
+  <si>
+    <t>連合会</t>
+  </si>
+  <si>
+    <t>れんごうかい</t>
+  </si>
+  <si>
+    <t>federasi, gabungan asosiasi</t>
+  </si>
+  <si>
+    <t>HP</t>
+  </si>
+  <si>
+    <t>エイチピー</t>
+  </si>
+  <si>
+    <t>homepage (situs web)</t>
   </si>
 </sst>
 </file>
@@ -6908,7 +7895,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G1118"/>
+  <dimension ref="A1:G1395"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="33" customWidth="1"/>
@@ -22641,6 +23628,3884 @@
         <v>868</v>
       </c>
     </row>
+    <row r="1119" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1119" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1119" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="C1119" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1119" s="12" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1120" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1120" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="C1120" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1120" s="12" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1121" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1121" s="12" t="s">
+        <v>2190</v>
+      </c>
+      <c r="C1121" s="12" t="s">
+        <v>2191</v>
+      </c>
+      <c r="D1121" s="12" t="s">
+        <v>2192</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1122" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1122" s="12" t="s">
+        <v>2193</v>
+      </c>
+      <c r="C1122" s="12" t="s">
+        <v>2193</v>
+      </c>
+      <c r="D1122" s="12" t="s">
+        <v>2194</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1123" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1123" s="12" t="s">
+        <v>538</v>
+      </c>
+      <c r="C1123" s="12" t="s">
+        <v>539</v>
+      </c>
+      <c r="D1123" s="12" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1124" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1124" s="12" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1124" s="12" t="s">
+        <v>503</v>
+      </c>
+      <c r="D1124" s="12" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1125" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1125" s="12" t="s">
+        <v>1385</v>
+      </c>
+      <c r="C1125" s="12" t="s">
+        <v>1386</v>
+      </c>
+      <c r="D1125" s="12" t="s">
+        <v>2195</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1126" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1126" s="12" t="s">
+        <v>2196</v>
+      </c>
+      <c r="C1126" s="12" t="s">
+        <v>2197</v>
+      </c>
+      <c r="D1126" s="12" t="s">
+        <v>2198</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1127" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1127" s="12" t="s">
+        <v>2199</v>
+      </c>
+      <c r="C1127" s="12" t="s">
+        <v>2200</v>
+      </c>
+      <c r="D1127" s="12" t="s">
+        <v>2201</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1128" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1128" s="12" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1128" s="12" t="s">
+        <v>1446</v>
+      </c>
+      <c r="D1128" s="12" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1129" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1129" s="12" t="s">
+        <v>2202</v>
+      </c>
+      <c r="C1129" s="12" t="s">
+        <v>2203</v>
+      </c>
+      <c r="D1129" s="12" t="s">
+        <v>2204</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1130" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1130" s="12" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1130" s="12" t="s">
+        <v>503</v>
+      </c>
+      <c r="D1130" s="12" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1131" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1131" s="12" t="s">
+        <v>1343</v>
+      </c>
+      <c r="C1131" s="12" t="s">
+        <v>1344</v>
+      </c>
+      <c r="D1131" s="12" t="s">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1132" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1132" s="12" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C1132" s="12" t="s">
+        <v>1081</v>
+      </c>
+      <c r="D1132" s="12" t="s">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1133" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1133" s="12" t="s">
+        <v>2206</v>
+      </c>
+      <c r="C1133" s="12" t="s">
+        <v>2207</v>
+      </c>
+      <c r="D1133" s="12" t="s">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1134" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1134" s="12" t="s">
+        <v>2209</v>
+      </c>
+      <c r="C1134" s="12" t="s">
+        <v>2210</v>
+      </c>
+      <c r="D1134" s="12" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1135" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1135" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="C1135" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="D1135" s="12" t="s">
+        <v>2212</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1136" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1136" s="12" t="s">
+        <v>2213</v>
+      </c>
+      <c r="C1136" s="12" t="s">
+        <v>2214</v>
+      </c>
+      <c r="D1136" s="12" t="s">
+        <v>2215</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1137" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1137" s="12" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C1137" s="12" t="s">
+        <v>1298</v>
+      </c>
+      <c r="D1137" s="12" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1138" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1138" s="12" t="s">
+        <v>2202</v>
+      </c>
+      <c r="C1138" s="12" t="s">
+        <v>2203</v>
+      </c>
+      <c r="D1138" s="12" t="s">
+        <v>2216</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1139" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1139" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="C1139" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1139" s="12" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="1140" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1140" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1140" s="12" t="s">
+        <v>2217</v>
+      </c>
+      <c r="C1140" s="12" t="s">
+        <v>2218</v>
+      </c>
+      <c r="D1140" s="12" t="s">
+        <v>2219</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1141" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1141" s="12" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1141" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="D1141" s="12" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1142" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1142" s="12" t="s">
+        <v>1988</v>
+      </c>
+      <c r="C1142" s="12" t="s">
+        <v>1989</v>
+      </c>
+      <c r="D1142" s="12" t="s">
+        <v>1990</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1143" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1143" s="12" t="s">
+        <v>2220</v>
+      </c>
+      <c r="C1143" s="12" t="s">
+        <v>2221</v>
+      </c>
+      <c r="D1143" s="12" t="s">
+        <v>2222</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1144" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1144" s="12" t="s">
+        <v>2223</v>
+      </c>
+      <c r="C1144" s="12" t="s">
+        <v>2224</v>
+      </c>
+      <c r="D1144" s="12" t="s">
+        <v>2225</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1145" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1145" s="12" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1145" s="12" t="s">
+        <v>503</v>
+      </c>
+      <c r="D1145" s="12" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1146" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1146" s="12" t="s">
+        <v>2226</v>
+      </c>
+      <c r="C1146" s="12" t="s">
+        <v>2226</v>
+      </c>
+      <c r="D1146" s="12" t="s">
+        <v>2227</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1147" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1147" s="12" t="s">
+        <v>1980</v>
+      </c>
+      <c r="C1147" s="12" t="s">
+        <v>1981</v>
+      </c>
+      <c r="D1147" s="12" t="s">
+        <v>1952</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1148" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1148" s="12" t="s">
+        <v>2228</v>
+      </c>
+      <c r="C1148" s="12" t="s">
+        <v>2229</v>
+      </c>
+      <c r="D1148" s="12" t="s">
+        <v>2230</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1149" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1149" s="12" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1149" s="12" t="s">
+        <v>1446</v>
+      </c>
+      <c r="D1149" s="12" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1150" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1150" s="12" t="s">
+        <v>942</v>
+      </c>
+      <c r="C1150" s="12" t="s">
+        <v>943</v>
+      </c>
+      <c r="D1150" s="12" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1151" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1151" s="12" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C1151" s="12" t="s">
+        <v>1298</v>
+      </c>
+      <c r="D1151" s="12" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1152" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1152" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="C1152" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1152" s="12" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1153" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1153" s="12" t="s">
+        <v>2231</v>
+      </c>
+      <c r="C1153" s="12" t="s">
+        <v>2232</v>
+      </c>
+      <c r="D1153" s="12" t="s">
+        <v>2233</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1154" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1154" s="12" t="s">
+        <v>1950</v>
+      </c>
+      <c r="C1154" s="12" t="s">
+        <v>1951</v>
+      </c>
+      <c r="D1154" s="12" t="s">
+        <v>1952</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1155" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1155" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="C1155" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1155" s="12" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1156" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1156" s="12" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1156" s="12" t="s">
+        <v>503</v>
+      </c>
+      <c r="D1156" s="12" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1157" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1157" s="12" t="s">
+        <v>2234</v>
+      </c>
+      <c r="C1157" s="12" t="s">
+        <v>2235</v>
+      </c>
+      <c r="D1157" s="12" t="s">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1158" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1158" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="C1158" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1158" s="12" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1159" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1159" s="12" t="s">
+        <v>2237</v>
+      </c>
+      <c r="C1159" s="12" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D1159" s="12" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1160" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1160" s="12" t="s">
+        <v>2240</v>
+      </c>
+      <c r="C1160" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="D1160" s="12" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1161" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1161" s="12" t="s">
+        <v>328</v>
+      </c>
+      <c r="C1161" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="D1161" s="12" t="s">
+        <v>1908</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1162" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1162" s="12" t="s">
+        <v>2242</v>
+      </c>
+      <c r="C1162" s="12" t="s">
+        <v>2243</v>
+      </c>
+      <c r="D1162" s="12" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1163" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1163" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="C1163" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="D1163" s="12" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1164" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1164" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="C1164" s="12" t="s">
+        <v>392</v>
+      </c>
+      <c r="D1164" s="12" t="s">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1165" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1165" s="12" t="s">
+        <v>1988</v>
+      </c>
+      <c r="C1165" s="12" t="s">
+        <v>1989</v>
+      </c>
+      <c r="D1165" s="12" t="s">
+        <v>1990</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1166" s="1">
+        <v>17</v>
+      </c>
+      <c r="B1166" s="12" t="s">
+        <v>2223</v>
+      </c>
+      <c r="C1166" s="12" t="s">
+        <v>2224</v>
+      </c>
+      <c r="D1166" s="12" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1167" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1167" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="C1167" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="D1167" s="12" t="s">
+        <v>2248</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1168" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1168" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="C1168" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="D1168" s="12" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1169" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1169" s="12" t="s">
+        <v>951</v>
+      </c>
+      <c r="C1169" s="12" t="s">
+        <v>952</v>
+      </c>
+      <c r="D1169" s="12" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1170" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1170" s="12" t="s">
+        <v>954</v>
+      </c>
+      <c r="C1170" s="12" t="s">
+        <v>955</v>
+      </c>
+      <c r="D1170" s="12" t="s">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1171" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1171" s="12" t="s">
+        <v>1910</v>
+      </c>
+      <c r="C1171" s="12" t="s">
+        <v>1911</v>
+      </c>
+      <c r="D1171" s="12" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1172" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1172" s="12" t="s">
+        <v>2013</v>
+      </c>
+      <c r="C1172" s="12" t="s">
+        <v>2014</v>
+      </c>
+      <c r="D1172" s="12" t="s">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1173" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1173" s="12" t="s">
+        <v>2252</v>
+      </c>
+      <c r="C1173" s="12" t="s">
+        <v>2253</v>
+      </c>
+      <c r="D1173" s="12" t="s">
+        <v>2254</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1174" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1174" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1174" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1174" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1175" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1175" s="12" t="s">
+        <v>1926</v>
+      </c>
+      <c r="C1175" s="12" t="s">
+        <v>1927</v>
+      </c>
+      <c r="D1175" s="12" t="s">
+        <v>1928</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1176" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1176" s="12" t="s">
+        <v>753</v>
+      </c>
+      <c r="C1176" s="12" t="s">
+        <v>754</v>
+      </c>
+      <c r="D1176" s="12" t="s">
+        <v>2255</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1177" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1177" s="12" t="s">
+        <v>1623</v>
+      </c>
+      <c r="C1177" s="12" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D1177" s="12" t="s">
+        <v>2056</v>
+      </c>
+    </row>
+    <row r="1178" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1178" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1178" s="12" t="s">
+        <v>1992</v>
+      </c>
+      <c r="C1178" s="12" t="s">
+        <v>1993</v>
+      </c>
+      <c r="D1178" s="12" t="s">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="1179" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1179" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1179" s="12" t="s">
+        <v>1944</v>
+      </c>
+      <c r="C1179" s="12" t="s">
+        <v>1945</v>
+      </c>
+      <c r="D1179" s="12" t="s">
+        <v>1946</v>
+      </c>
+    </row>
+    <row r="1180" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1180" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1180" s="12" t="s">
+        <v>2256</v>
+      </c>
+      <c r="C1180" s="12" t="s">
+        <v>2257</v>
+      </c>
+      <c r="D1180" s="12" t="s">
+        <v>2258</v>
+      </c>
+    </row>
+    <row r="1181" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1181" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1181" s="12" t="s">
+        <v>1959</v>
+      </c>
+      <c r="C1181" s="12" t="s">
+        <v>1960</v>
+      </c>
+      <c r="D1181" s="12" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1182" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1182" s="12" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C1182" s="12" t="s">
+        <v>1313</v>
+      </c>
+      <c r="D1182" s="12" t="s">
+        <v>1970</v>
+      </c>
+    </row>
+    <row r="1183" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1183" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1183" s="12" t="s">
+        <v>2259</v>
+      </c>
+      <c r="C1183" s="12" t="s">
+        <v>2260</v>
+      </c>
+      <c r="D1183" s="12" t="s">
+        <v>2261</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1184" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1184" s="12" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C1184" s="12" t="s">
+        <v>1313</v>
+      </c>
+      <c r="D1184" s="12" t="s">
+        <v>1970</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1185" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1185" s="12" t="s">
+        <v>2262</v>
+      </c>
+      <c r="C1185" s="12" t="s">
+        <v>2263</v>
+      </c>
+      <c r="D1185" s="12" t="s">
+        <v>2264</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1186" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1186" s="12" t="s">
+        <v>1959</v>
+      </c>
+      <c r="C1186" s="12" t="s">
+        <v>1960</v>
+      </c>
+      <c r="D1186" s="12" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1187" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1187" s="12" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C1187" s="12" t="s">
+        <v>1313</v>
+      </c>
+      <c r="D1187" s="12" t="s">
+        <v>1970</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1188" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1188" s="12" t="s">
+        <v>1966</v>
+      </c>
+      <c r="C1188" s="12" t="s">
+        <v>1967</v>
+      </c>
+      <c r="D1188" s="12" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1189" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1189" s="12" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C1189" s="12" t="s">
+        <v>1313</v>
+      </c>
+      <c r="D1189" s="12" t="s">
+        <v>1970</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1190" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1190" s="12" t="s">
+        <v>2256</v>
+      </c>
+      <c r="C1190" s="12" t="s">
+        <v>2257</v>
+      </c>
+      <c r="D1190" s="12" t="s">
+        <v>2258</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1191" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1191" s="12" t="s">
+        <v>656</v>
+      </c>
+      <c r="C1191" s="12" t="s">
+        <v>657</v>
+      </c>
+      <c r="D1191" s="12" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1192" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1192" s="12" t="s">
+        <v>2115</v>
+      </c>
+      <c r="C1192" s="12" t="s">
+        <v>2116</v>
+      </c>
+      <c r="D1192" s="12" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1193" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1193" s="12" t="s">
+        <v>1959</v>
+      </c>
+      <c r="C1193" s="12" t="s">
+        <v>1960</v>
+      </c>
+      <c r="D1193" s="12" t="s">
+        <v>1961</v>
+      </c>
+    </row>
+    <row r="1194" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1194" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1194" s="12" t="s">
+        <v>1962</v>
+      </c>
+      <c r="C1194" s="12" t="s">
+        <v>1963</v>
+      </c>
+      <c r="D1194" s="12" t="s">
+        <v>1964</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1195" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1195" s="12" t="s">
+        <v>2265</v>
+      </c>
+      <c r="C1195" s="12" t="s">
+        <v>2266</v>
+      </c>
+      <c r="D1195" s="12" t="s">
+        <v>2267</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1196" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1196" s="12" t="s">
+        <v>1966</v>
+      </c>
+      <c r="C1196" s="12" t="s">
+        <v>1967</v>
+      </c>
+      <c r="D1196" s="12" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="1197" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1197" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1197" s="12" t="s">
+        <v>1962</v>
+      </c>
+      <c r="C1197" s="12" t="s">
+        <v>1963</v>
+      </c>
+      <c r="D1197" s="12" t="s">
+        <v>1964</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1198" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1198" s="12" t="s">
+        <v>2268</v>
+      </c>
+      <c r="C1198" s="12" t="s">
+        <v>2269</v>
+      </c>
+      <c r="D1198" s="12" t="s">
+        <v>2270</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1199" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1199" s="12" t="s">
+        <v>954</v>
+      </c>
+      <c r="C1199" s="12" t="s">
+        <v>955</v>
+      </c>
+      <c r="D1199" s="12" t="s">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1200" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1200" s="12" t="s">
+        <v>2271</v>
+      </c>
+      <c r="C1200" s="12" t="s">
+        <v>2272</v>
+      </c>
+      <c r="D1200" s="12" t="s">
+        <v>2273</v>
+      </c>
+    </row>
+    <row r="1201" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1201" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1201" s="12" t="s">
+        <v>2274</v>
+      </c>
+      <c r="C1201" s="12" t="s">
+        <v>2275</v>
+      </c>
+      <c r="D1201" s="12" t="s">
+        <v>2276</v>
+      </c>
+    </row>
+    <row r="1202" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1202" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1202" s="12" t="s">
+        <v>951</v>
+      </c>
+      <c r="C1202" s="12" t="s">
+        <v>952</v>
+      </c>
+      <c r="D1202" s="12" t="s">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="1203" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1203" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1203" s="12" t="s">
+        <v>1910</v>
+      </c>
+      <c r="C1203" s="12" t="s">
+        <v>1911</v>
+      </c>
+      <c r="D1203" s="12" t="s">
+        <v>2277</v>
+      </c>
+    </row>
+    <row r="1204" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1204" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1204" s="12" t="s">
+        <v>2278</v>
+      </c>
+      <c r="C1204" s="12" t="s">
+        <v>2279</v>
+      </c>
+      <c r="D1204" s="12" t="s">
+        <v>2280</v>
+      </c>
+    </row>
+    <row r="1205" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1205" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1205" s="12" t="s">
+        <v>2281</v>
+      </c>
+      <c r="C1205" s="12" t="s">
+        <v>2282</v>
+      </c>
+      <c r="D1205" s="12" t="s">
+        <v>2283</v>
+      </c>
+    </row>
+    <row r="1206" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1206" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1206" s="12" t="s">
+        <v>2284</v>
+      </c>
+      <c r="C1206" s="12" t="s">
+        <v>2285</v>
+      </c>
+      <c r="D1206" s="12" t="s">
+        <v>2286</v>
+      </c>
+    </row>
+    <row r="1207" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1207" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1207" s="12" t="s">
+        <v>2287</v>
+      </c>
+      <c r="C1207" s="12" t="s">
+        <v>2288</v>
+      </c>
+      <c r="D1207" s="12" t="s">
+        <v>2289</v>
+      </c>
+    </row>
+    <row r="1208" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1208" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1208" s="12" t="s">
+        <v>2290</v>
+      </c>
+      <c r="C1208" s="12" t="s">
+        <v>2291</v>
+      </c>
+      <c r="D1208" s="12" t="s">
+        <v>2292</v>
+      </c>
+    </row>
+    <row r="1209" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1209" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1209" s="12" t="s">
+        <v>2293</v>
+      </c>
+      <c r="C1209" s="12" t="s">
+        <v>2294</v>
+      </c>
+      <c r="D1209" s="12" t="s">
+        <v>2295</v>
+      </c>
+    </row>
+    <row r="1210" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1210" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1210" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1210" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1210" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1211" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1211" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1211" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="C1211" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="D1211" s="12" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="1212" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1212" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1212" s="12" t="s">
+        <v>2209</v>
+      </c>
+      <c r="C1212" s="12" t="s">
+        <v>2210</v>
+      </c>
+      <c r="D1212" s="12" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="1213" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1213" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1213" s="12" t="s">
+        <v>1926</v>
+      </c>
+      <c r="C1213" s="12" t="s">
+        <v>1927</v>
+      </c>
+      <c r="D1213" s="12" t="s">
+        <v>1928</v>
+      </c>
+    </row>
+    <row r="1214" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1214" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1214" s="12" t="s">
+        <v>2296</v>
+      </c>
+      <c r="C1214" s="12" t="s">
+        <v>2297</v>
+      </c>
+      <c r="D1214" s="12" t="s">
+        <v>2298</v>
+      </c>
+    </row>
+    <row r="1215" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1215" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1215" s="12" t="s">
+        <v>2299</v>
+      </c>
+      <c r="C1215" s="12" t="s">
+        <v>2300</v>
+      </c>
+      <c r="D1215" s="12" t="s">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="1216" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1216" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1216" s="12" t="s">
+        <v>2302</v>
+      </c>
+      <c r="C1216" s="12" t="s">
+        <v>2303</v>
+      </c>
+      <c r="D1216" s="12" t="s">
+        <v>2304</v>
+      </c>
+    </row>
+    <row r="1217" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1217" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1217" s="12" t="s">
+        <v>2305</v>
+      </c>
+      <c r="C1217" s="12" t="s">
+        <v>2306</v>
+      </c>
+      <c r="D1217" s="12" t="s">
+        <v>2307</v>
+      </c>
+    </row>
+    <row r="1218" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1218" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1218" s="12" t="s">
+        <v>1274</v>
+      </c>
+      <c r="C1218" s="12" t="s">
+        <v>1275</v>
+      </c>
+      <c r="D1218" s="12" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="1219" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1219" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1219" s="12" t="s">
+        <v>1283</v>
+      </c>
+      <c r="C1219" s="12" t="s">
+        <v>1284</v>
+      </c>
+      <c r="D1219" s="12" t="s">
+        <v>2308</v>
+      </c>
+    </row>
+    <row r="1220" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1220" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1220" s="12" t="s">
+        <v>2309</v>
+      </c>
+      <c r="C1220" s="12" t="s">
+        <v>2310</v>
+      </c>
+      <c r="D1220" s="12" t="s">
+        <v>2311</v>
+      </c>
+    </row>
+    <row r="1221" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1221" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1221" s="12" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C1221" s="12" t="s">
+        <v>1298</v>
+      </c>
+      <c r="D1221" s="12" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="1222" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1222" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1222" s="12" t="s">
+        <v>2209</v>
+      </c>
+      <c r="C1222" s="12" t="s">
+        <v>2210</v>
+      </c>
+      <c r="D1222" s="12" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="1223" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1223" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1223" s="12" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1223" s="12" t="s">
+        <v>1446</v>
+      </c>
+      <c r="D1223" s="12" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="1224" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1224" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1224" s="12" t="s">
+        <v>2312</v>
+      </c>
+      <c r="C1224" s="12" t="s">
+        <v>2313</v>
+      </c>
+      <c r="D1224" s="12" t="s">
+        <v>2314</v>
+      </c>
+    </row>
+    <row r="1225" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1225" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1225" s="12" t="s">
+        <v>2315</v>
+      </c>
+      <c r="C1225" s="12" t="s">
+        <v>2316</v>
+      </c>
+      <c r="D1225" s="12" t="s">
+        <v>2317</v>
+      </c>
+    </row>
+    <row r="1226" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1226" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1226" s="12" t="s">
+        <v>2318</v>
+      </c>
+      <c r="C1226" s="12" t="s">
+        <v>2319</v>
+      </c>
+      <c r="D1226" s="12" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="1227" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1227" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1227" s="12" t="s">
+        <v>2320</v>
+      </c>
+      <c r="C1227" s="12" t="s">
+        <v>2321</v>
+      </c>
+      <c r="D1227" s="12" t="s">
+        <v>2322</v>
+      </c>
+    </row>
+    <row r="1228" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1228" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1228" s="12" t="s">
+        <v>2323</v>
+      </c>
+      <c r="C1228" s="12" t="s">
+        <v>2324</v>
+      </c>
+      <c r="D1228" s="12" t="s">
+        <v>2325</v>
+      </c>
+    </row>
+    <row r="1229" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1229" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1229" s="12" t="s">
+        <v>2326</v>
+      </c>
+      <c r="C1229" s="12" t="s">
+        <v>2327</v>
+      </c>
+      <c r="D1229" s="12" t="s">
+        <v>2328</v>
+      </c>
+    </row>
+    <row r="1230" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1230" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1230" s="12" t="s">
+        <v>524</v>
+      </c>
+      <c r="C1230" s="12" t="s">
+        <v>525</v>
+      </c>
+      <c r="D1230" s="12" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1231" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1231" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1231" s="12" t="s">
+        <v>2281</v>
+      </c>
+      <c r="C1231" s="12" t="s">
+        <v>2282</v>
+      </c>
+      <c r="D1231" s="12" t="s">
+        <v>2283</v>
+      </c>
+    </row>
+    <row r="1232" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1232" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1232" s="12" t="s">
+        <v>2329</v>
+      </c>
+      <c r="C1232" s="12" t="s">
+        <v>2330</v>
+      </c>
+      <c r="D1232" s="12" t="s">
+        <v>2331</v>
+      </c>
+    </row>
+    <row r="1233" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1233" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1233" s="12" t="s">
+        <v>2046</v>
+      </c>
+      <c r="C1233" s="12" t="s">
+        <v>2047</v>
+      </c>
+      <c r="D1233" s="12" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="1234" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1234" s="1">
+        <v>18</v>
+      </c>
+      <c r="B1234" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1234" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1234" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1235" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1235" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1235" s="12" t="s">
+        <v>2332</v>
+      </c>
+      <c r="C1235" s="12" t="s">
+        <v>2333</v>
+      </c>
+      <c r="D1235" s="12" t="s">
+        <v>2334</v>
+      </c>
+    </row>
+    <row r="1236" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1236" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1236" s="12" t="s">
+        <v>2332</v>
+      </c>
+      <c r="C1236" s="12" t="s">
+        <v>2333</v>
+      </c>
+      <c r="D1236" s="12" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1237" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1237" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1237" s="12" t="s">
+        <v>2312</v>
+      </c>
+      <c r="C1237" s="12" t="s">
+        <v>2313</v>
+      </c>
+      <c r="D1237" s="12" t="s">
+        <v>2336</v>
+      </c>
+    </row>
+    <row r="1238" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1238" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1238" s="12" t="s">
+        <v>2337</v>
+      </c>
+      <c r="C1238" s="12" t="s">
+        <v>2338</v>
+      </c>
+      <c r="D1238" s="12" t="s">
+        <v>2339</v>
+      </c>
+    </row>
+    <row r="1239" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1239" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1239" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="C1239" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1239" s="12" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="1240" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1240" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1240" s="12" t="s">
+        <v>2013</v>
+      </c>
+      <c r="C1240" s="12" t="s">
+        <v>2014</v>
+      </c>
+      <c r="D1240" s="12" t="s">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="1241" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1241" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1241" s="12" t="s">
+        <v>2340</v>
+      </c>
+      <c r="C1241" s="12" t="s">
+        <v>2341</v>
+      </c>
+      <c r="D1241" s="12" t="s">
+        <v>2342</v>
+      </c>
+    </row>
+    <row r="1242" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1242" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1242" s="12" t="s">
+        <v>1920</v>
+      </c>
+      <c r="C1242" s="12" t="s">
+        <v>1921</v>
+      </c>
+      <c r="D1242" s="12" t="s">
+        <v>1922</v>
+      </c>
+    </row>
+    <row r="1243" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1243" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1243" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1243" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1243" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1244" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1244" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1244" s="12" t="s">
+        <v>2332</v>
+      </c>
+      <c r="C1244" s="12" t="s">
+        <v>2333</v>
+      </c>
+      <c r="D1244" s="12" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1245" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1245" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1245" s="12" t="s">
+        <v>2318</v>
+      </c>
+      <c r="C1245" s="12" t="s">
+        <v>2319</v>
+      </c>
+      <c r="D1245" s="12" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="1246" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1246" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1246" s="12" t="s">
+        <v>2320</v>
+      </c>
+      <c r="C1246" s="12" t="s">
+        <v>2321</v>
+      </c>
+      <c r="D1246" s="12" t="s">
+        <v>2322</v>
+      </c>
+    </row>
+    <row r="1247" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1247" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1247" s="12" t="s">
+        <v>2323</v>
+      </c>
+      <c r="C1247" s="12" t="s">
+        <v>2324</v>
+      </c>
+      <c r="D1247" s="12" t="s">
+        <v>2325</v>
+      </c>
+    </row>
+    <row r="1248" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1248" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1248" s="12" t="s">
+        <v>2343</v>
+      </c>
+      <c r="C1248" s="12" t="s">
+        <v>2344</v>
+      </c>
+      <c r="D1248" s="12" t="s">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="1249" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1249" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1249" s="12" t="s">
+        <v>2332</v>
+      </c>
+      <c r="C1249" s="12" t="s">
+        <v>2333</v>
+      </c>
+      <c r="D1249" s="12" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1250" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1250" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1250" s="12" t="s">
+        <v>2343</v>
+      </c>
+      <c r="C1250" s="12" t="s">
+        <v>2344</v>
+      </c>
+      <c r="D1250" s="12" t="s">
+        <v>2346</v>
+      </c>
+    </row>
+    <row r="1251" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1251" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1251" s="12" t="s">
+        <v>2318</v>
+      </c>
+      <c r="C1251" s="12" t="s">
+        <v>2319</v>
+      </c>
+      <c r="D1251" s="12" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="1252" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1252" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1252" s="12" t="s">
+        <v>2347</v>
+      </c>
+      <c r="C1252" s="12" t="s">
+        <v>2348</v>
+      </c>
+      <c r="D1252" s="12" t="s">
+        <v>2349</v>
+      </c>
+    </row>
+    <row r="1253" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1253" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1253" s="12" t="s">
+        <v>2350</v>
+      </c>
+      <c r="C1253" s="12" t="s">
+        <v>2351</v>
+      </c>
+      <c r="D1253" s="12" t="s">
+        <v>2352</v>
+      </c>
+    </row>
+    <row r="1254" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1254" s="1">
+        <v>19</v>
+      </c>
+      <c r="B1254" s="12" t="s">
+        <v>2353</v>
+      </c>
+      <c r="C1254" s="12" t="s">
+        <v>2354</v>
+      </c>
+      <c r="D1254" s="12" t="s">
+        <v>2355</v>
+      </c>
+    </row>
+    <row r="1255" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1255" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1255" s="12" t="s">
+        <v>483</v>
+      </c>
+      <c r="C1255" s="12" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1255" s="12" t="s">
+        <v>2356</v>
+      </c>
+    </row>
+    <row r="1256" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1256" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1256" s="12" t="s">
+        <v>483</v>
+      </c>
+      <c r="C1256" s="12" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1256" s="12" t="s">
+        <v>2357</v>
+      </c>
+    </row>
+    <row r="1257" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1257" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1257" s="12" t="s">
+        <v>2358</v>
+      </c>
+      <c r="C1257" s="12" t="s">
+        <v>2359</v>
+      </c>
+      <c r="D1257" s="12" t="s">
+        <v>2360</v>
+      </c>
+    </row>
+    <row r="1258" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1258" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1258" s="12" t="s">
+        <v>2361</v>
+      </c>
+      <c r="C1258" s="12" t="s">
+        <v>2362</v>
+      </c>
+      <c r="D1258" s="12" t="s">
+        <v>2363</v>
+      </c>
+    </row>
+    <row r="1259" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1259" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1259" s="12" t="s">
+        <v>948</v>
+      </c>
+      <c r="C1259" s="12" t="s">
+        <v>949</v>
+      </c>
+      <c r="D1259" s="12" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="1260" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1260" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1260" s="12" t="s">
+        <v>2364</v>
+      </c>
+      <c r="C1260" s="12" t="s">
+        <v>2365</v>
+      </c>
+      <c r="D1260" s="12" t="s">
+        <v>2366</v>
+      </c>
+    </row>
+    <row r="1261" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1261" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1261" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="C1261" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="D1261" s="12" t="s">
+        <v>2212</v>
+      </c>
+    </row>
+    <row r="1262" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1262" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1262" s="12" t="s">
+        <v>2367</v>
+      </c>
+      <c r="C1262" s="12" t="s">
+        <v>2368</v>
+      </c>
+      <c r="D1262" s="12" t="s">
+        <v>2369</v>
+      </c>
+    </row>
+    <row r="1263" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1263" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1263" s="12" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C1263" s="12" t="s">
+        <v>1446</v>
+      </c>
+      <c r="D1263" s="12" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="1264" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1264" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1264" s="12" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C1264" s="12" t="s">
+        <v>1194</v>
+      </c>
+      <c r="D1264" s="12" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="1265" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1265" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1265" s="12" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C1265" s="12" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D1265" s="12" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="1266" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1266" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1266" s="12" t="s">
+        <v>948</v>
+      </c>
+      <c r="C1266" s="12" t="s">
+        <v>949</v>
+      </c>
+      <c r="D1266" s="12" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="1267" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1267" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1267" s="12" t="s">
+        <v>2370</v>
+      </c>
+      <c r="C1267" s="12" t="s">
+        <v>2203</v>
+      </c>
+      <c r="D1267" s="12" t="s">
+        <v>2371</v>
+      </c>
+    </row>
+    <row r="1268" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1268" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1268" s="12" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C1268" s="12" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D1268" s="12" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="1269" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1269" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1269" s="12" t="s">
+        <v>2281</v>
+      </c>
+      <c r="C1269" s="12" t="s">
+        <v>2282</v>
+      </c>
+      <c r="D1269" s="12" t="s">
+        <v>2283</v>
+      </c>
+    </row>
+    <row r="1270" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1270" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1270" s="12" t="s">
+        <v>2372</v>
+      </c>
+      <c r="C1270" s="12" t="s">
+        <v>2373</v>
+      </c>
+      <c r="D1270" s="12" t="s">
+        <v>2006</v>
+      </c>
+    </row>
+    <row r="1271" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1271" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1271" s="12" t="s">
+        <v>2374</v>
+      </c>
+      <c r="C1271" s="12" t="s">
+        <v>2375</v>
+      </c>
+      <c r="D1271" s="12" t="s">
+        <v>2376</v>
+      </c>
+    </row>
+    <row r="1272" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1272" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1272" s="12" t="s">
+        <v>2377</v>
+      </c>
+      <c r="C1272" s="12" t="s">
+        <v>2378</v>
+      </c>
+      <c r="D1272" s="12" t="s">
+        <v>2379</v>
+      </c>
+    </row>
+    <row r="1273" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1273" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1273" s="12" t="s">
+        <v>2380</v>
+      </c>
+      <c r="C1273" s="12" t="s">
+        <v>2381</v>
+      </c>
+      <c r="D1273" s="12" t="s">
+        <v>2382</v>
+      </c>
+    </row>
+    <row r="1274" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1274" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1274" s="12" t="s">
+        <v>1920</v>
+      </c>
+      <c r="C1274" s="12" t="s">
+        <v>1921</v>
+      </c>
+      <c r="D1274" s="12" t="s">
+        <v>1922</v>
+      </c>
+    </row>
+    <row r="1275" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1275" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1275" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="C1275" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="D1275" s="12" t="s">
+        <v>2383</v>
+      </c>
+    </row>
+    <row r="1276" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1276" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1276" s="12" t="s">
+        <v>2374</v>
+      </c>
+      <c r="C1276" s="12" t="s">
+        <v>2375</v>
+      </c>
+      <c r="D1276" s="12" t="s">
+        <v>2376</v>
+      </c>
+    </row>
+    <row r="1277" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1277" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1277" s="12" t="s">
+        <v>2384</v>
+      </c>
+      <c r="C1277" s="12" t="s">
+        <v>2385</v>
+      </c>
+      <c r="D1277" s="12" t="s">
+        <v>2386</v>
+      </c>
+    </row>
+    <row r="1278" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1278" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1278" s="12" t="s">
+        <v>2387</v>
+      </c>
+      <c r="C1278" s="12" t="s">
+        <v>2388</v>
+      </c>
+      <c r="D1278" s="12" t="s">
+        <v>2389</v>
+      </c>
+    </row>
+    <row r="1279" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1279" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1279" s="12" t="s">
+        <v>2007</v>
+      </c>
+      <c r="C1279" s="12" t="s">
+        <v>2008</v>
+      </c>
+      <c r="D1279" s="12" t="s">
+        <v>2009</v>
+      </c>
+    </row>
+    <row r="1280" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1280" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1280" s="12" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C1280" s="12" t="s">
+        <v>2391</v>
+      </c>
+      <c r="D1280" s="12" t="s">
+        <v>2392</v>
+      </c>
+    </row>
+    <row r="1281" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1281" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1281" s="12" t="s">
+        <v>2393</v>
+      </c>
+      <c r="C1281" s="12" t="s">
+        <v>2394</v>
+      </c>
+      <c r="D1281" s="12" t="s">
+        <v>2395</v>
+      </c>
+    </row>
+    <row r="1282" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1282" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1282" s="12" t="s">
+        <v>2374</v>
+      </c>
+      <c r="C1282" s="12" t="s">
+        <v>2375</v>
+      </c>
+      <c r="D1282" s="12" t="s">
+        <v>2376</v>
+      </c>
+    </row>
+    <row r="1283" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1283" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1283" s="12" t="s">
+        <v>1049</v>
+      </c>
+      <c r="C1283" s="12" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D1283" s="12" t="s">
+        <v>2396</v>
+      </c>
+    </row>
+    <row r="1284" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1284" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1284" s="12" t="s">
+        <v>1926</v>
+      </c>
+      <c r="C1284" s="12" t="s">
+        <v>1927</v>
+      </c>
+      <c r="D1284" s="12" t="s">
+        <v>1928</v>
+      </c>
+    </row>
+    <row r="1285" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1285" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1285" s="12" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C1285" s="12" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D1285" s="12" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="1286" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1286" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1286" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="C1286" s="12" t="s">
+        <v>543</v>
+      </c>
+      <c r="D1286" s="12" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1287" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1287" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1287" s="12" t="s">
+        <v>2397</v>
+      </c>
+      <c r="C1287" s="12" t="s">
+        <v>2398</v>
+      </c>
+      <c r="D1287" s="12" t="s">
+        <v>2399</v>
+      </c>
+    </row>
+    <row r="1288" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1288" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1288" s="12" t="s">
+        <v>564</v>
+      </c>
+      <c r="C1288" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="D1288" s="12" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="1289" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1289" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1289" s="12" t="s">
+        <v>987</v>
+      </c>
+      <c r="C1289" s="12" t="s">
+        <v>988</v>
+      </c>
+      <c r="D1289" s="12" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="1290" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1290" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1290" s="12" t="s">
+        <v>2400</v>
+      </c>
+      <c r="C1290" s="12" t="s">
+        <v>2401</v>
+      </c>
+      <c r="D1290" s="12" t="s">
+        <v>2298</v>
+      </c>
+    </row>
+    <row r="1291" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1291" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1291" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="C1291" s="12" t="s">
+        <v>543</v>
+      </c>
+      <c r="D1291" s="12" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1292" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1292" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1292" s="12" t="s">
+        <v>1920</v>
+      </c>
+      <c r="C1292" s="12" t="s">
+        <v>1921</v>
+      </c>
+      <c r="D1292" s="12" t="s">
+        <v>1922</v>
+      </c>
+    </row>
+    <row r="1293" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1293" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1293" s="12" t="s">
+        <v>2402</v>
+      </c>
+      <c r="C1293" s="12" t="s">
+        <v>2403</v>
+      </c>
+      <c r="D1293" s="12" t="s">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="1294" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1294" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1294" s="12" t="s">
+        <v>907</v>
+      </c>
+      <c r="C1294" s="12" t="s">
+        <v>908</v>
+      </c>
+      <c r="D1294" s="12" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="1295" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1295" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1295" s="12" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C1295" s="12" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D1295" s="12" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="1296" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1296" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1296" s="12" t="s">
+        <v>2405</v>
+      </c>
+      <c r="C1296" s="12" t="s">
+        <v>2406</v>
+      </c>
+      <c r="D1296" s="12" t="s">
+        <v>2407</v>
+      </c>
+    </row>
+    <row r="1297" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1297" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1297" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1297" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1297" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1298" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1298" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1298" s="12" t="s">
+        <v>483</v>
+      </c>
+      <c r="C1298" s="12" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1298" s="12" t="s">
+        <v>2408</v>
+      </c>
+    </row>
+    <row r="1299" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1299" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1299" s="12" t="s">
+        <v>675</v>
+      </c>
+      <c r="C1299" s="12" t="s">
+        <v>676</v>
+      </c>
+      <c r="D1299" s="12" t="s">
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="1300" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1300" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1300" s="12" t="s">
+        <v>2409</v>
+      </c>
+      <c r="C1300" s="12" t="s">
+        <v>2410</v>
+      </c>
+      <c r="D1300" s="12" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="1301" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1301" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1301" s="12" t="s">
+        <v>2411</v>
+      </c>
+      <c r="C1301" s="12" t="s">
+        <v>2412</v>
+      </c>
+      <c r="D1301" s="12" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="1302" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1302" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1302" s="12" t="s">
+        <v>907</v>
+      </c>
+      <c r="C1302" s="12" t="s">
+        <v>908</v>
+      </c>
+      <c r="D1302" s="12" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="1303" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1303" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1303" s="12" t="s">
+        <v>866</v>
+      </c>
+      <c r="C1303" s="12" t="s">
+        <v>867</v>
+      </c>
+      <c r="D1303" s="12" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="1304" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1304" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1304" s="12" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1304" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="D1304" s="12" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1305" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1305" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1305" s="12" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C1305" s="12" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D1305" s="12" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="1306" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1306" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1306" s="12" t="s">
+        <v>934</v>
+      </c>
+      <c r="C1306" s="12" t="s">
+        <v>935</v>
+      </c>
+      <c r="D1306" s="12" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="1307" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1307" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1307" s="12" t="s">
+        <v>888</v>
+      </c>
+      <c r="C1307" s="12" t="s">
+        <v>889</v>
+      </c>
+      <c r="D1307" s="12" t="s">
+        <v>2413</v>
+      </c>
+    </row>
+    <row r="1308" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1308" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1308" s="12" t="s">
+        <v>2414</v>
+      </c>
+      <c r="C1308" s="12" t="s">
+        <v>2415</v>
+      </c>
+      <c r="D1308" s="12" t="s">
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="1309" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1309" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1309" s="12" t="s">
+        <v>866</v>
+      </c>
+      <c r="C1309" s="12" t="s">
+        <v>867</v>
+      </c>
+      <c r="D1309" s="12" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="1310" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1310" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1310" s="12" t="s">
+        <v>2397</v>
+      </c>
+      <c r="C1310" s="12" t="s">
+        <v>2398</v>
+      </c>
+      <c r="D1310" s="12" t="s">
+        <v>2417</v>
+      </c>
+    </row>
+    <row r="1311" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1311" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1311" s="12" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1311" s="12" t="s">
+        <v>1316</v>
+      </c>
+      <c r="D1311" s="12" t="s">
+        <v>2418</v>
+      </c>
+    </row>
+    <row r="1312" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1312" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1312" s="12" t="s">
+        <v>2419</v>
+      </c>
+      <c r="C1312" s="12" t="s">
+        <v>2420</v>
+      </c>
+      <c r="D1312" s="12" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="1313" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1313" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1313" s="12" t="s">
+        <v>2421</v>
+      </c>
+      <c r="C1313" s="12" t="s">
+        <v>2422</v>
+      </c>
+      <c r="D1313" s="12" t="s">
+        <v>2423</v>
+      </c>
+    </row>
+    <row r="1314" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1314" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1314" s="12" t="s">
+        <v>2424</v>
+      </c>
+      <c r="C1314" s="12" t="s">
+        <v>2425</v>
+      </c>
+      <c r="D1314" s="12" t="s">
+        <v>2426</v>
+      </c>
+    </row>
+    <row r="1315" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1315" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1315" s="12" t="s">
+        <v>2427</v>
+      </c>
+      <c r="C1315" s="12" t="s">
+        <v>2428</v>
+      </c>
+      <c r="D1315" s="12" t="s">
+        <v>2429</v>
+      </c>
+    </row>
+    <row r="1316" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1316" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1316" s="12" t="s">
+        <v>2430</v>
+      </c>
+      <c r="C1316" s="12" t="s">
+        <v>2431</v>
+      </c>
+      <c r="D1316" s="12" t="s">
+        <v>2432</v>
+      </c>
+    </row>
+    <row r="1317" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1317" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1317" s="12" t="s">
+        <v>2433</v>
+      </c>
+      <c r="C1317" s="12" t="s">
+        <v>2434</v>
+      </c>
+      <c r="D1317" s="12" t="s">
+        <v>2435</v>
+      </c>
+    </row>
+    <row r="1318" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1318" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1318" s="12" t="s">
+        <v>2436</v>
+      </c>
+      <c r="C1318" s="12" t="s">
+        <v>2437</v>
+      </c>
+      <c r="D1318" s="12" t="s">
+        <v>2438</v>
+      </c>
+    </row>
+    <row r="1319" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1319" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1319" s="12" t="s">
+        <v>2439</v>
+      </c>
+      <c r="C1319" s="12" t="s">
+        <v>2440</v>
+      </c>
+      <c r="D1319" s="12" t="s">
+        <v>2441</v>
+      </c>
+    </row>
+    <row r="1320" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1320" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1320" s="12" t="s">
+        <v>552</v>
+      </c>
+      <c r="C1320" s="12" t="s">
+        <v>553</v>
+      </c>
+      <c r="D1320" s="12" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="1321" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1321" s="1">
+        <v>20</v>
+      </c>
+      <c r="B1321" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1321" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1321" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1322" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1322" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1322" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1322" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="D1322" s="12" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1323" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1323" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1323" s="12" t="s">
+        <v>2442</v>
+      </c>
+      <c r="C1323" s="12" t="s">
+        <v>2443</v>
+      </c>
+      <c r="D1323" s="12" t="s">
+        <v>2444</v>
+      </c>
+    </row>
+    <row r="1324" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1324" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1324" s="12" t="s">
+        <v>2445</v>
+      </c>
+      <c r="C1324" s="12" t="s">
+        <v>2446</v>
+      </c>
+      <c r="D1324" s="12" t="s">
+        <v>2447</v>
+      </c>
+    </row>
+    <row r="1325" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1325" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1325" s="12" t="s">
+        <v>2318</v>
+      </c>
+      <c r="C1325" s="12" t="s">
+        <v>2319</v>
+      </c>
+      <c r="D1325" s="12" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="1326" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1326" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1326" s="12" t="s">
+        <v>2448</v>
+      </c>
+      <c r="C1326" s="12" t="s">
+        <v>2449</v>
+      </c>
+      <c r="D1326" s="12" t="s">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="1327" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1327" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1327" s="12" t="s">
+        <v>483</v>
+      </c>
+      <c r="C1327" s="12" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1327" s="12" t="s">
+        <v>2356</v>
+      </c>
+    </row>
+    <row r="1328" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1328" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1328" s="12" t="s">
+        <v>2318</v>
+      </c>
+      <c r="C1328" s="12" t="s">
+        <v>2319</v>
+      </c>
+      <c r="D1328" s="12" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="1329" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1329" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1329" s="12" t="s">
+        <v>2451</v>
+      </c>
+      <c r="C1329" s="12" t="s">
+        <v>2452</v>
+      </c>
+      <c r="D1329" s="12" t="s">
+        <v>2453</v>
+      </c>
+    </row>
+    <row r="1330" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1330" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1330" s="12" t="s">
+        <v>2454</v>
+      </c>
+      <c r="C1330" s="12" t="s">
+        <v>2455</v>
+      </c>
+      <c r="D1330" s="12" t="s">
+        <v>2456</v>
+      </c>
+    </row>
+    <row r="1331" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1331" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1331" s="12" t="s">
+        <v>2457</v>
+      </c>
+      <c r="C1331" s="12" t="s">
+        <v>2458</v>
+      </c>
+      <c r="D1331" s="12" t="s">
+        <v>2459</v>
+      </c>
+    </row>
+    <row r="1332" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1332" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1332" s="12" t="s">
+        <v>2397</v>
+      </c>
+      <c r="C1332" s="12" t="s">
+        <v>2398</v>
+      </c>
+      <c r="D1332" s="12" t="s">
+        <v>2399</v>
+      </c>
+    </row>
+    <row r="1333" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1333" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1333" s="12" t="s">
+        <v>564</v>
+      </c>
+      <c r="C1333" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="D1333" s="12" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="1334" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1334" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1334" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1334" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1334" s="12" t="s">
+        <v>2006</v>
+      </c>
+    </row>
+    <row r="1335" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1335" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1335" s="12" t="s">
+        <v>2460</v>
+      </c>
+      <c r="C1335" s="12" t="s">
+        <v>2461</v>
+      </c>
+      <c r="D1335" s="12" t="s">
+        <v>2462</v>
+      </c>
+    </row>
+    <row r="1336" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1336" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1336" s="12" t="s">
+        <v>1808</v>
+      </c>
+      <c r="C1336" s="12" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D1336" s="12" t="s">
+        <v>1783</v>
+      </c>
+    </row>
+    <row r="1337" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1337" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1337" s="12" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C1337" s="12" t="s">
+        <v>1377</v>
+      </c>
+      <c r="D1337" s="12" t="s">
+        <v>2463</v>
+      </c>
+    </row>
+    <row r="1338" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1338" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1338" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1338" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1338" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1339" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1339" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1339" s="12" t="s">
+        <v>483</v>
+      </c>
+      <c r="C1339" s="12" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1339" s="12" t="s">
+        <v>2357</v>
+      </c>
+    </row>
+    <row r="1340" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1340" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1340" s="12" t="s">
+        <v>524</v>
+      </c>
+      <c r="C1340" s="12" t="s">
+        <v>525</v>
+      </c>
+      <c r="D1340" s="12" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1341" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1341" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1341" s="12" t="s">
+        <v>2003</v>
+      </c>
+      <c r="C1341" s="12" t="s">
+        <v>2004</v>
+      </c>
+      <c r="D1341" s="12" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="1342" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1342" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1342" s="12" t="s">
+        <v>1871</v>
+      </c>
+      <c r="C1342" s="12" t="s">
+        <v>1872</v>
+      </c>
+      <c r="D1342" s="12" t="s">
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="1343" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1343" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1343" s="12" t="s">
+        <v>2086</v>
+      </c>
+      <c r="C1343" s="12" t="s">
+        <v>2087</v>
+      </c>
+      <c r="D1343" s="12" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="1344" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1344" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1344" s="12" t="s">
+        <v>2464</v>
+      </c>
+      <c r="C1344" s="12" t="s">
+        <v>2465</v>
+      </c>
+      <c r="D1344" s="12" t="s">
+        <v>2466</v>
+      </c>
+    </row>
+    <row r="1345" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1345" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1345" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1345" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1345" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1346" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1346" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1346" s="12" t="s">
+        <v>558</v>
+      </c>
+      <c r="C1346" s="12" t="s">
+        <v>559</v>
+      </c>
+      <c r="D1346" s="12" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="1347" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1347" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1347" s="12" t="s">
+        <v>2467</v>
+      </c>
+      <c r="C1347" s="12" t="s">
+        <v>2468</v>
+      </c>
+      <c r="D1347" s="12" t="s">
+        <v>2469</v>
+      </c>
+    </row>
+    <row r="1348" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1348" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1348" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1348" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1348" s="12" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="1349" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1349" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1349" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="C1349" s="12" t="s">
+        <v>543</v>
+      </c>
+      <c r="D1349" s="12" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1350" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1350" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1350" s="12" t="s">
+        <v>1171</v>
+      </c>
+      <c r="C1350" s="12" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D1350" s="12" t="s">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="1351" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1351" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1351" s="12" t="s">
+        <v>866</v>
+      </c>
+      <c r="C1351" s="12" t="s">
+        <v>867</v>
+      </c>
+      <c r="D1351" s="12" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="1352" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1352" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1352" s="12" t="s">
+        <v>733</v>
+      </c>
+      <c r="C1352" s="12" t="s">
+        <v>734</v>
+      </c>
+      <c r="D1352" s="12" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="1353" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1353" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1353" s="12" t="s">
+        <v>2470</v>
+      </c>
+      <c r="C1353" s="12" t="s">
+        <v>2471</v>
+      </c>
+      <c r="D1353" s="12" t="s">
+        <v>2472</v>
+      </c>
+    </row>
+    <row r="1354" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1354" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1354" s="12" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1354" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="D1354" s="12" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1355" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1355" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1355" s="12" t="s">
+        <v>907</v>
+      </c>
+      <c r="C1355" s="12" t="s">
+        <v>908</v>
+      </c>
+      <c r="D1355" s="12" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="1356" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1356" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1356" s="12" t="s">
+        <v>2003</v>
+      </c>
+      <c r="C1356" s="12" t="s">
+        <v>2004</v>
+      </c>
+      <c r="D1356" s="12" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="1357" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1357" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1357" s="12" t="s">
+        <v>1871</v>
+      </c>
+      <c r="C1357" s="12" t="s">
+        <v>1872</v>
+      </c>
+      <c r="D1357" s="12" t="s">
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="1358" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1358" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1358" s="12" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C1358" s="12" t="s">
+        <v>1154</v>
+      </c>
+      <c r="D1358" s="12" t="s">
+        <v>1155</v>
+      </c>
+    </row>
+    <row r="1359" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1359" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1359" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1359" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1359" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1360" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1360" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1360" s="12" t="s">
+        <v>1561</v>
+      </c>
+      <c r="C1360" s="12" t="s">
+        <v>1562</v>
+      </c>
+      <c r="D1360" s="12" t="s">
+        <v>2473</v>
+      </c>
+    </row>
+    <row r="1361" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1361" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1361" s="12" t="s">
+        <v>2474</v>
+      </c>
+      <c r="C1361" s="12" t="s">
+        <v>2475</v>
+      </c>
+      <c r="D1361" s="12" t="s">
+        <v>2476</v>
+      </c>
+    </row>
+    <row r="1362" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1362" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1362" s="12" t="s">
+        <v>866</v>
+      </c>
+      <c r="C1362" s="12" t="s">
+        <v>867</v>
+      </c>
+      <c r="D1362" s="12" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="1363" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1363" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1363" s="12" t="s">
+        <v>1871</v>
+      </c>
+      <c r="C1363" s="12" t="s">
+        <v>1872</v>
+      </c>
+      <c r="D1363" s="12" t="s">
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="1364" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1364" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1364" s="12" t="s">
+        <v>2150</v>
+      </c>
+      <c r="C1364" s="12" t="s">
+        <v>2151</v>
+      </c>
+      <c r="D1364" s="12" t="s">
+        <v>2477</v>
+      </c>
+    </row>
+    <row r="1365" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1365" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1365" s="12" t="s">
+        <v>2478</v>
+      </c>
+      <c r="C1365" s="12" t="s">
+        <v>2479</v>
+      </c>
+      <c r="D1365" s="12" t="s">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="1366" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1366" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1366" s="12" t="s">
+        <v>2470</v>
+      </c>
+      <c r="C1366" s="12" t="s">
+        <v>2471</v>
+      </c>
+      <c r="D1366" s="12" t="s">
+        <v>2472</v>
+      </c>
+    </row>
+    <row r="1367" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1367" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1367" s="12" t="s">
+        <v>2481</v>
+      </c>
+      <c r="C1367" s="12" t="s">
+        <v>2482</v>
+      </c>
+      <c r="D1367" s="12" t="s">
+        <v>2483</v>
+      </c>
+    </row>
+    <row r="1368" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1368" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1368" s="12" t="s">
+        <v>1926</v>
+      </c>
+      <c r="C1368" s="12" t="s">
+        <v>1927</v>
+      </c>
+      <c r="D1368" s="12" t="s">
+        <v>1928</v>
+      </c>
+    </row>
+    <row r="1369" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1369" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1369" s="12" t="s">
+        <v>2484</v>
+      </c>
+      <c r="C1369" s="12" t="s">
+        <v>2485</v>
+      </c>
+      <c r="D1369" s="12" t="s">
+        <v>2486</v>
+      </c>
+    </row>
+    <row r="1370" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1370" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1370" s="12" t="s">
+        <v>987</v>
+      </c>
+      <c r="C1370" s="12" t="s">
+        <v>988</v>
+      </c>
+      <c r="D1370" s="12" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="1371" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1371" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1371" s="12" t="s">
+        <v>2063</v>
+      </c>
+      <c r="C1371" s="12" t="s">
+        <v>2064</v>
+      </c>
+      <c r="D1371" s="12" t="s">
+        <v>2487</v>
+      </c>
+    </row>
+    <row r="1372" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1372" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1372" s="12" t="s">
+        <v>2063</v>
+      </c>
+      <c r="C1372" s="12" t="s">
+        <v>2064</v>
+      </c>
+      <c r="D1372" s="12" t="s">
+        <v>2487</v>
+      </c>
+    </row>
+    <row r="1373" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1373" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1373" s="12" t="s">
+        <v>2066</v>
+      </c>
+      <c r="C1373" s="12" t="s">
+        <v>2067</v>
+      </c>
+      <c r="D1373" s="12" t="s">
+        <v>2068</v>
+      </c>
+    </row>
+    <row r="1374" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1374" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1374" s="12" t="s">
+        <v>2488</v>
+      </c>
+      <c r="C1374" s="12" t="s">
+        <v>2489</v>
+      </c>
+      <c r="D1374" s="12" t="s">
+        <v>2490</v>
+      </c>
+    </row>
+    <row r="1375" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1375" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1375" s="12" t="s">
+        <v>2491</v>
+      </c>
+      <c r="C1375" s="12" t="s">
+        <v>2492</v>
+      </c>
+      <c r="D1375" s="12" t="s">
+        <v>2493</v>
+      </c>
+    </row>
+    <row r="1376" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1376" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1376" s="12" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C1376" s="12" t="s">
+        <v>1096</v>
+      </c>
+      <c r="D1376" s="12" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="1377" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1377" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1377" s="12" t="s">
+        <v>2400</v>
+      </c>
+      <c r="C1377" s="12" t="s">
+        <v>2401</v>
+      </c>
+      <c r="D1377" s="12" t="s">
+        <v>2298</v>
+      </c>
+    </row>
+    <row r="1378" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1378" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1378" s="12" t="s">
+        <v>907</v>
+      </c>
+      <c r="C1378" s="12" t="s">
+        <v>908</v>
+      </c>
+      <c r="D1378" s="12" t="s">
+        <v>2495</v>
+      </c>
+    </row>
+    <row r="1379" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1379" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1379" s="12" t="s">
+        <v>2003</v>
+      </c>
+      <c r="C1379" s="12" t="s">
+        <v>2004</v>
+      </c>
+      <c r="D1379" s="12" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="1380" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1380" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1380" s="12" t="s">
+        <v>1871</v>
+      </c>
+      <c r="C1380" s="12" t="s">
+        <v>1872</v>
+      </c>
+      <c r="D1380" s="12" t="s">
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="1381" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1381" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1381" s="12" t="s">
+        <v>2086</v>
+      </c>
+      <c r="C1381" s="12" t="s">
+        <v>2087</v>
+      </c>
+      <c r="D1381" s="12" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="1382" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1382" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1382" s="12" t="s">
+        <v>2464</v>
+      </c>
+      <c r="C1382" s="12" t="s">
+        <v>2465</v>
+      </c>
+      <c r="D1382" s="12" t="s">
+        <v>2496</v>
+      </c>
+    </row>
+    <row r="1383" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1383" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1383" s="12" t="s">
+        <v>2063</v>
+      </c>
+      <c r="C1383" s="12" t="s">
+        <v>2064</v>
+      </c>
+      <c r="D1383" s="12" t="s">
+        <v>2497</v>
+      </c>
+    </row>
+    <row r="1384" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1384" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1384" s="12" t="s">
+        <v>2491</v>
+      </c>
+      <c r="C1384" s="12" t="s">
+        <v>2492</v>
+      </c>
+      <c r="D1384" s="12" t="s">
+        <v>2493</v>
+      </c>
+    </row>
+    <row r="1385" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1385" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1385" s="12" t="s">
+        <v>2095</v>
+      </c>
+      <c r="C1385" s="12" t="s">
+        <v>2096</v>
+      </c>
+      <c r="D1385" s="12" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="1386" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1386" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1386" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1386" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D1386" s="12" t="s">
+        <v>2498</v>
+      </c>
+    </row>
+    <row r="1387" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1387" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1387" s="12" t="s">
+        <v>564</v>
+      </c>
+      <c r="C1387" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="D1387" s="12" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="1388" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1388" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1388" s="12" t="s">
+        <v>2499</v>
+      </c>
+      <c r="C1388" s="12" t="s">
+        <v>2500</v>
+      </c>
+      <c r="D1388" s="12" t="s">
+        <v>2501</v>
+      </c>
+    </row>
+    <row r="1389" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1389" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1389" s="12" t="s">
+        <v>2502</v>
+      </c>
+      <c r="C1389" s="12" t="s">
+        <v>2503</v>
+      </c>
+      <c r="D1389" s="12" t="s">
+        <v>2504</v>
+      </c>
+    </row>
+    <row r="1390" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1390" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1390" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1390" s="12" t="s">
+        <v>609</v>
+      </c>
+      <c r="D1390" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="1391" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1391" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1391" s="12" t="s">
+        <v>483</v>
+      </c>
+      <c r="C1391" s="12" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1391" s="12" t="s">
+        <v>2356</v>
+      </c>
+    </row>
+    <row r="1392" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1392" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1392" s="12" t="s">
+        <v>2505</v>
+      </c>
+      <c r="C1392" s="12" t="s">
+        <v>2506</v>
+      </c>
+      <c r="D1392" s="12" t="s">
+        <v>2507</v>
+      </c>
+    </row>
+    <row r="1393" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1393" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1393" s="12" t="s">
+        <v>2508</v>
+      </c>
+      <c r="C1393" s="12" t="s">
+        <v>2509</v>
+      </c>
+      <c r="D1393" s="12" t="s">
+        <v>2510</v>
+      </c>
+    </row>
+    <row r="1394" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1394" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1394" s="12" t="s">
+        <v>2511</v>
+      </c>
+      <c r="C1394" s="12" t="s">
+        <v>2512</v>
+      </c>
+      <c r="D1394" s="12" t="s">
+        <v>2513</v>
+      </c>
+    </row>
+    <row r="1395" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A1395" s="1">
+        <v>21</v>
+      </c>
+      <c r="B1395" s="12" t="s">
+        <v>2514</v>
+      </c>
+      <c r="C1395" s="12" t="s">
+        <v>2515</v>
+      </c>
+      <c r="D1395" s="12" t="s">
+        <v>2516</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>